<commit_message>
updated last week details
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -25,7 +25,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ ddd"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
@@ -36,6 +36,7 @@
     <numFmt numFmtId="171" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="172" formatCode="#,##0.##;\(#,##0.##\);&quot;-&quot;"/>
     <numFmt numFmtId="173" formatCode="#,##0;\-#,##0;\-"/>
+    <numFmt numFmtId="174" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="86">
     <font>
@@ -8286,17 +8287,46 @@
       <c r="Q32" s="44" t="n"/>
     </row>
     <row r="33" ht="16.5" customHeight="1" s="274">
-      <c r="B33" s="34" t="n"/>
-      <c r="C33" s="47" t="n"/>
-      <c r="D33" s="48" t="n"/>
-      <c r="E33" s="49" t="n"/>
-      <c r="F33" s="50" t="n"/>
-      <c r="G33" s="51" t="n"/>
-      <c r="H33" s="52" t="n"/>
-      <c r="I33" s="53" t="n"/>
-      <c r="J33" s="54" t="n"/>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>12-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D33" s="48" t="n">
+        <v>2635</v>
+      </c>
+      <c r="E33" s="49" t="n">
+        <v>3435</v>
+      </c>
+      <c r="F33" s="50">
+        <f>IFERROR(D33+E33+G33,0)</f>
+        <v/>
+      </c>
+      <c r="G33" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="52" t="n">
+        <v>901.8</v>
+      </c>
+      <c r="I33" s="53">
+        <f>IFERROR(F33-H33,0)</f>
+        <v/>
+      </c>
+      <c r="J33" s="54">
+        <f>IFERROR(I33/F33,0)</f>
+        <v/>
+      </c>
       <c r="K33" s="55" t="n"/>
-      <c r="L33" s="18" t="n"/>
+      <c r="L33" s="18" t="inlineStr">
+        <is>
+          <t>Cierre 12 Jun + receipts</t>
+        </is>
+      </c>
       <c r="M33" s="21" t="n"/>
       <c r="N33" s="56" t="n"/>
       <c r="O33" s="57" t="n"/>
@@ -8304,17 +8334,46 @@
       <c r="Q33" s="56" t="n"/>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="274">
-      <c r="B34" s="34" t="n"/>
-      <c r="C34" s="35" t="n"/>
-      <c r="D34" s="36" t="n"/>
-      <c r="E34" s="37" t="n"/>
-      <c r="F34" s="38" t="n"/>
-      <c r="G34" s="39" t="n"/>
-      <c r="H34" s="40" t="n"/>
-      <c r="I34" s="41" t="n"/>
-      <c r="J34" s="42" t="n"/>
+      <c r="B34" s="34" t="inlineStr">
+        <is>
+          <t>13-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C34" s="35" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D34" s="36" t="n">
+        <v>1005</v>
+      </c>
+      <c r="E34" s="37" t="n">
+        <v>806</v>
+      </c>
+      <c r="F34" s="38">
+        <f>IFERROR(D34+E34+G34,0)</f>
+        <v/>
+      </c>
+      <c r="G34" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="40" t="n">
+        <v>778.16</v>
+      </c>
+      <c r="I34" s="41">
+        <f>IFERROR(F34-H34,0)</f>
+        <v/>
+      </c>
+      <c r="J34" s="42">
+        <f>IFERROR(I34/F34,0)</f>
+        <v/>
+      </c>
       <c r="K34" s="43" t="n"/>
-      <c r="L34" s="9" t="n"/>
+      <c r="L34" s="9" t="inlineStr">
+        <is>
+          <t>Cierre 13 Jun + receipts</t>
+        </is>
+      </c>
       <c r="M34" s="12" t="n"/>
       <c r="N34" s="44" t="n"/>
       <c r="O34" s="45" t="n"/>
@@ -14407,9 +14466,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -24298,7 +24357,7 @@
       </c>
       <c r="G241" s="23" t="inlineStr">
         <is>
-          <t>Restaurant</t>
+          <t>Lohith (Personal)</t>
         </is>
       </c>
       <c r="H241" s="23" t="inlineStr">
@@ -24313,7 +24372,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>Paid cash exact $2,865 · 08:22 AM</t>
+          <t>Paid cash exact $2,865 · 08:22 AM | Paid personally by Lohith (transfer) — reimburse</t>
         </is>
       </c>
     </row>
@@ -24341,7 +24400,7 @@
       </c>
       <c r="G242" s="14" t="inlineStr">
         <is>
-          <t>Restaurant</t>
+          <t>Lohith (Personal)</t>
         </is>
       </c>
       <c r="H242" s="14" t="inlineStr">
@@ -24356,7 +24415,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>Pink nota "Oh Lele" · marked Cobrado</t>
+          <t>Pink nota "Oh Lele" · marked Cobrado | Paid personally by Lohith (transfer) — reimburse</t>
         </is>
       </c>
     </row>
@@ -24490,74 +24549,305 @@
       </c>
     </row>
     <row r="246">
-      <c r="B246" s="64" t="n"/>
-      <c r="C246" s="65" t="n"/>
-      <c r="D246" s="66" t="n"/>
-      <c r="E246" s="65" t="n"/>
-      <c r="F246" s="67" t="n"/>
-      <c r="G246" s="14" t="n"/>
-      <c r="H246" s="14" t="n"/>
-      <c r="I246" s="43" t="n"/>
+      <c r="B246" s="64" t="n">
+        <v>46185</v>
+      </c>
+      <c r="C246" s="65" t="inlineStr">
+        <is>
+          <t>Leche PL UHT Nutri 1LT (2 pcs)</t>
+        </is>
+      </c>
+      <c r="D246" s="66" t="inlineStr">
+        <is>
+          <t>OXXO Acueducto</t>
+        </is>
+      </c>
+      <c r="E246" s="65" t="inlineStr">
+        <is>
+          <t>Ingredients - Dairy</t>
+        </is>
+      </c>
+      <c r="F246" s="67" t="n">
+        <v>42</v>
+      </c>
+      <c r="G246" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H246" s="14" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I246" s="43" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>ML debit **3982 · Aut 324051 · 10:13</t>
+        </is>
+      </c>
     </row>
     <row r="247">
-      <c r="B247" s="64" t="n"/>
-      <c r="C247" s="69" t="n"/>
-      <c r="D247" s="68" t="n"/>
-      <c r="E247" s="69" t="n"/>
-      <c r="F247" s="70" t="n"/>
-      <c r="G247" s="23" t="n"/>
-      <c r="H247" s="23" t="n"/>
-      <c r="I247" s="55" t="n"/>
+      <c r="B247" s="64" t="n">
+        <v>46185</v>
+      </c>
+      <c r="C247" s="69" t="inlineStr">
+        <is>
+          <t>Pan hamburguesa ajonjolí (36) + Chapata grande (24)</t>
+        </is>
+      </c>
+      <c r="D247" s="68" t="inlineStr">
+        <is>
+          <t>Productos Real (La Cruz)</t>
+        </is>
+      </c>
+      <c r="E247" s="69" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F247" s="70" t="n">
+        <v>546</v>
+      </c>
+      <c r="G247" s="23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H247" s="23" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I247" s="55" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Folio 4251 · debit · 09:38</t>
+        </is>
+      </c>
     </row>
     <row r="248">
-      <c r="B248" s="64" t="n"/>
-      <c r="C248" s="65" t="n"/>
-      <c r="D248" s="66" t="n"/>
-      <c r="E248" s="65" t="n"/>
-      <c r="F248" s="67" t="n"/>
-      <c r="G248" s="14" t="n"/>
-      <c r="H248" s="14" t="n"/>
-      <c r="I248" s="43" t="n"/>
+      <c r="B248" s="64" t="n">
+        <v>46185</v>
+      </c>
+      <c r="C248" s="65" t="inlineStr">
+        <is>
+          <t>Aceite Vegetal La Posada 800 (2 pcs)</t>
+        </is>
+      </c>
+      <c r="D248" s="66" t="inlineStr">
+        <is>
+          <t>OXXO Pathe</t>
+        </is>
+      </c>
+      <c r="E248" s="65" t="inlineStr">
+        <is>
+          <t>Ingredients - Other</t>
+        </is>
+      </c>
+      <c r="F248" s="67" t="n">
+        <v>104</v>
+      </c>
+      <c r="G248" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H248" s="14" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I248" s="43" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>ML debit **3982 · Aut 468013 · 09:22</t>
+        </is>
+      </c>
     </row>
     <row r="249">
-      <c r="B249" s="64" t="n"/>
-      <c r="C249" s="69" t="n"/>
-      <c r="D249" s="68" t="n"/>
-      <c r="E249" s="69" t="n"/>
-      <c r="F249" s="70" t="n"/>
-      <c r="G249" s="23" t="n"/>
-      <c r="H249" s="23" t="n"/>
-      <c r="I249" s="55" t="n"/>
+      <c r="B249" s="64" t="n">
+        <v>46185</v>
+      </c>
+      <c r="C249" s="69" t="inlineStr">
+        <is>
+          <t>Plátano + Tortillas Blancas + Rosca Marmoleada</t>
+        </is>
+      </c>
+      <c r="D249" s="68" t="inlineStr">
+        <is>
+          <t>Chedraui Paseo</t>
+        </is>
+      </c>
+      <c r="E249" s="69" t="inlineStr">
+        <is>
+          <t>Supermarket / General</t>
+        </is>
+      </c>
+      <c r="F249" s="70" t="n">
+        <v>161.8</v>
+      </c>
+      <c r="G249" s="23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H249" s="23" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I249" s="55" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Debit BBVA **3982 · Aut 200580 · 09:02</t>
+        </is>
+      </c>
     </row>
     <row r="250">
-      <c r="B250" s="64" t="n"/>
-      <c r="C250" s="65" t="n"/>
-      <c r="D250" s="66" t="n"/>
-      <c r="E250" s="65" t="n"/>
-      <c r="F250" s="67" t="n"/>
-      <c r="G250" s="14" t="n"/>
-      <c r="H250" s="14" t="n"/>
-      <c r="I250" s="43" t="n"/>
+      <c r="B250" s="64" t="n">
+        <v>46185</v>
+      </c>
+      <c r="C250" s="65" t="inlineStr">
+        <is>
+          <t>Lechugas (lettuce)</t>
+        </is>
+      </c>
+      <c r="D250" s="66" t="inlineStr">
+        <is>
+          <t>Local purchase</t>
+        </is>
+      </c>
+      <c r="E250" s="65" t="inlineStr">
+        <is>
+          <t>Ingredients - Produce</t>
+        </is>
+      </c>
+      <c r="F250" s="67" t="n">
+        <v>48</v>
+      </c>
+      <c r="G250" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H250" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I250" s="43" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>No receipt — logged manually</t>
+        </is>
+      </c>
     </row>
     <row r="251">
-      <c r="B251" s="64" t="n"/>
-      <c r="C251" s="69" t="n"/>
-      <c r="D251" s="68" t="n"/>
-      <c r="E251" s="69" t="n"/>
-      <c r="F251" s="70" t="n"/>
-      <c r="G251" s="23" t="n"/>
-      <c r="H251" s="23" t="n"/>
-      <c r="I251" s="55" t="n"/>
+      <c r="B251" s="64" t="n">
+        <v>46186</v>
+      </c>
+      <c r="C251" s="69" t="inlineStr">
+        <is>
+          <t>Empanizador Bimbo, especias, tomate, pimiento verde, papa, mole, tortillas (14 art.)</t>
+        </is>
+      </c>
+      <c r="D251" s="68" t="inlineStr">
+        <is>
+          <t>Chedraui Paseo</t>
+        </is>
+      </c>
+      <c r="E251" s="69" t="inlineStr">
+        <is>
+          <t>Supermarket / General</t>
+        </is>
+      </c>
+      <c r="F251" s="70" t="n">
+        <v>468.16</v>
+      </c>
+      <c r="G251" s="23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H251" s="23" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I251" s="55" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Debit BBVA **3982 · Aut 641502 · 09:19 · Folio 2606-1309-1901</t>
+        </is>
+      </c>
     </row>
     <row r="252">
-      <c r="B252" s="64" t="n"/>
-      <c r="C252" s="65" t="n"/>
-      <c r="D252" s="66" t="n"/>
-      <c r="E252" s="65" t="n"/>
-      <c r="F252" s="67" t="n"/>
-      <c r="G252" s="14" t="n"/>
-      <c r="H252" s="14" t="n"/>
-      <c r="I252" s="43" t="n"/>
+      <c r="B252" s="64" t="n">
+        <v>46186</v>
+      </c>
+      <c r="C252" s="65" t="inlineStr">
+        <is>
+          <t>Bistec de Cerdo 1.66 kg</t>
+        </is>
+      </c>
+      <c r="D252" s="66" t="inlineStr">
+        <is>
+          <t>Carnicería (nota de remisión)</t>
+        </is>
+      </c>
+      <c r="E252" s="65" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F252" s="67" t="n">
+        <v>310</v>
+      </c>
+      <c r="G252" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H252" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I252" s="43" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Handwritten remisión · 1.66 kg · total $310</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="B253" s="64" t="n"/>
@@ -30742,7 +31032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="18.33203125" customWidth="1" style="274" min="1" max="1"/>
@@ -32441,62 +32731,99 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="226" t="inlineStr">
+      <c r="A74" s="265" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B74" s="266" t="inlineStr">
+        <is>
+          <t>ALICO — Ala de Pollo, Papa Harvest 13.62kg, Boneless Freskecito</t>
+        </is>
+      </c>
+      <c r="C74" s="267" t="inlineStr">
+        <is>
+          <t>Expense - Personal</t>
+        </is>
+      </c>
+      <c r="D74" s="268" t="n">
+        <v>2865</v>
+      </c>
+      <c r="F74" s="269">
+        <f>IFERROR(F73+D74-E74,0)</f>
+        <v/>
+      </c>
+      <c r="G74" s="266" t="inlineStr">
+        <is>
+          <t>⏳ Reimburse</t>
+        </is>
+      </c>
+      <c r="H74" s="242" t="inlineStr">
+        <is>
+          <t>Restaurant ingredients paid personally by Lohith (transfer) — 11 Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="265" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B75" s="266" t="inlineStr">
+        <is>
+          <t>Pollería — Muslo de Pollo 4.70 kg</t>
+        </is>
+      </c>
+      <c r="C75" s="267" t="inlineStr">
+        <is>
+          <t>Expense - Personal</t>
+        </is>
+      </c>
+      <c r="D75" s="268" t="n">
+        <v>235</v>
+      </c>
+      <c r="F75" s="269">
+        <f>IFERROR(F74+D75-E75,0)</f>
+        <v/>
+      </c>
+      <c r="G75" s="266" t="inlineStr">
+        <is>
+          <t>⏳ Reimburse</t>
+        </is>
+      </c>
+      <c r="H75" s="242" t="inlineStr">
+        <is>
+          <t>Restaurant ingredients paid personally by Lohith (transfer) — 11 Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="226" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B74" s="219" t="n"/>
-      <c r="C74" s="219" t="n"/>
-      <c r="D74" s="256">
-        <f>SUM(D63:D73)</f>
-        <v/>
-      </c>
-      <c r="E74" s="257">
-        <f>SUM(E63:E73)</f>
-        <v/>
-      </c>
-      <c r="F74" s="258">
-        <f>F73</f>
-        <v/>
-      </c>
-      <c r="G74" s="226">
-        <f>IF(F73&gt;0,"⏳ Restaurant owes Lohith $"&amp;TEXT(F73,"#,##0"),IF(F73&lt;0,"💵 Lohith holds $"&amp;TEXT(ABS(F73),"#,##0"),"✅ Zero balance"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="242" t="inlineStr">
-        <is>
-          <t>HOW TO USE:</t>
-        </is>
-      </c>
-      <c r="B76" s="242" t="n"/>
-      <c r="C76" s="242" t="n"/>
-      <c r="D76" s="242" t="n"/>
-      <c r="E76" s="242" t="n"/>
-      <c r="F76" s="242" t="n"/>
-      <c r="G76" s="242" t="n"/>
-      <c r="H76" s="242" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="242" t="inlineStr">
-        <is>
-          <t>Add new rows above TOTALS. Spent by Lohith = restaurant expenses he paid personally.</t>
-        </is>
-      </c>
-      <c r="B77" s="242" t="n"/>
-      <c r="C77" s="242" t="n"/>
-      <c r="D77" s="242" t="n"/>
-      <c r="E77" s="242" t="n"/>
-      <c r="F77" s="242" t="n"/>
-      <c r="G77" s="242" t="n"/>
-      <c r="H77" s="242" t="n"/>
-    </row>
+      <c r="B76" s="219" t="n"/>
+      <c r="C76" s="219" t="n"/>
+      <c r="D76" s="256">
+        <f>SUM(D63:D75)</f>
+        <v/>
+      </c>
+      <c r="E76" s="257">
+        <f>SUM(E63:E75)</f>
+        <v/>
+      </c>
+      <c r="F76" s="258">
+        <f>F75</f>
+        <v/>
+      </c>
+      <c r="G76" s="226">
+        <f>IF(F75&gt;0,"⏳ Restaurant owes Lohith $"&amp;TEXT(F75,"#,##0"),IF(F75&lt;0,"💵 Lohith holds $"&amp;TEXT(ABS(F75),"#,##0"),"✅ Zero balance"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="242" t="inlineStr">
         <is>
-          <t>Transferred to Lohith = customer bank transfers received in his personal account.</t>
+          <t>HOW TO USE:</t>
         </is>
       </c>
       <c r="B78" s="242" t="n"/>
@@ -32510,7 +32837,7 @@
     <row r="79">
       <c r="A79" s="242" t="inlineStr">
         <is>
-          <t>Positive balance = restaurant owes Lohith. Negative = Lohith holds restaurant funds.</t>
+          <t>Add new rows above TOTALS. Spent by Lohith = restaurant expenses he paid personally.</t>
         </is>
       </c>
       <c r="B79" s="242" t="n"/>
@@ -32520,6 +32847,34 @@
       <c r="F79" s="242" t="n"/>
       <c r="G79" s="242" t="n"/>
       <c r="H79" s="242" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="242" t="inlineStr">
+        <is>
+          <t>Transferred to Lohith = customer bank transfers received in his personal account.</t>
+        </is>
+      </c>
+      <c r="B80" s="242" t="n"/>
+      <c r="C80" s="242" t="n"/>
+      <c r="D80" s="242" t="n"/>
+      <c r="E80" s="242" t="n"/>
+      <c r="F80" s="242" t="n"/>
+      <c r="G80" s="242" t="n"/>
+      <c r="H80" s="242" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="242" t="inlineStr">
+        <is>
+          <t>Positive balance = restaurant owes Lohith. Negative = Lohith holds restaurant funds.</t>
+        </is>
+      </c>
+      <c r="B81" s="242" t="n"/>
+      <c r="C81" s="242" t="n"/>
+      <c r="D81" s="242" t="n"/>
+      <c r="E81" s="242" t="n"/>
+      <c r="F81" s="242" t="n"/>
+      <c r="G81" s="242" t="n"/>
+      <c r="H81" s="242" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
updated todays expenses so far
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -9445,17 +9445,39 @@
       <c r="Q37" s="56" t="n"/>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="274">
-      <c r="B38" s="34" t="n"/>
-      <c r="C38" s="35" t="n"/>
+      <c r="B38" s="356" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C38" s="35" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
       <c r="D38" s="36" t="n"/>
       <c r="E38" s="37" t="n"/>
-      <c r="F38" s="38" t="n"/>
+      <c r="F38" s="38">
+        <f>IFERROR(D38+E38+G38,0)</f>
+        <v/>
+      </c>
       <c r="G38" s="39" t="n"/>
-      <c r="H38" s="40" t="n"/>
-      <c r="I38" s="41" t="n"/>
-      <c r="J38" s="42" t="n"/>
+      <c r="H38" s="40">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B38,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B38+1))</f>
+        <v/>
+      </c>
+      <c r="I38" s="41">
+        <f>IFERROR(F38-H38,0)</f>
+        <v/>
+      </c>
+      <c r="J38" s="42">
+        <f>IFERROR(I38/F38,0)</f>
+        <v/>
+      </c>
       <c r="K38" s="43" t="n"/>
-      <c r="L38" s="9" t="n"/>
+      <c r="L38" s="9" t="inlineStr">
+        <is>
+          <t>Expenses logged — revenue pending</t>
+        </is>
+      </c>
       <c r="M38" s="12" t="n"/>
       <c r="N38" s="44" t="n"/>
       <c r="O38" s="45" t="n"/>
@@ -15476,8 +15498,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -26935,54 +26957,219 @@
       </c>
     </row>
     <row r="278">
-      <c r="B278" s="64" t="n"/>
-      <c r="C278" s="69" t="n"/>
-      <c r="D278" s="68" t="n"/>
-      <c r="E278" s="69" t="n"/>
-      <c r="F278" s="70" t="n"/>
-      <c r="G278" s="23" t="n"/>
-      <c r="H278" s="23" t="n"/>
-      <c r="I278" s="55" t="n"/>
+      <c r="B278" s="64" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C278" s="69" t="inlineStr">
+        <is>
+          <t>Jamaica 1LT (6) + Té Fresco 1LT (6) — 12 pzas</t>
+        </is>
+      </c>
+      <c r="D278" s="68" t="inlineStr">
+        <is>
+          <t>Casa Reca</t>
+        </is>
+      </c>
+      <c r="E278" s="69" t="inlineStr">
+        <is>
+          <t>Ingredients - Beverages</t>
+        </is>
+      </c>
+      <c r="F278" s="70" t="n">
+        <v>300</v>
+      </c>
+      <c r="G278" s="23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H278" s="23" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I278" s="55" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Nota QR-3 · Café Oh lele</t>
+        </is>
+      </c>
     </row>
     <row r="279">
-      <c r="B279" s="64" t="n"/>
-      <c r="C279" s="65" t="n"/>
-      <c r="D279" s="66" t="n"/>
-      <c r="E279" s="65" t="n"/>
-      <c r="F279" s="67" t="n"/>
-      <c r="G279" s="14" t="n"/>
-      <c r="H279" s="14" t="n"/>
-      <c r="I279" s="43" t="n"/>
+      <c r="B279" s="64" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C279" s="65" t="inlineStr">
+        <is>
+          <t>Bolsas papel #5/#6, Vasos plást. 4CH, Tapas</t>
+        </is>
+      </c>
+      <c r="D279" s="66" t="inlineStr">
+        <is>
+          <t>Guimar Polietilenos</t>
+        </is>
+      </c>
+      <c r="E279" s="65" t="inlineStr">
+        <is>
+          <t>Supplies / Other</t>
+        </is>
+      </c>
+      <c r="F279" s="67" t="n">
+        <v>173</v>
+      </c>
+      <c r="G279" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H279" s="14" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I279" s="43" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Débito **28 · Folio XCC37437</t>
+        </is>
+      </c>
     </row>
     <row r="280">
-      <c r="B280" s="64" t="n"/>
-      <c r="C280" s="69" t="n"/>
-      <c r="D280" s="68" t="n"/>
-      <c r="E280" s="69" t="n"/>
-      <c r="F280" s="70" t="n"/>
-      <c r="G280" s="23" t="n"/>
-      <c r="H280" s="23" t="n"/>
-      <c r="I280" s="55" t="n"/>
+      <c r="B280" s="64" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C280" s="69" t="inlineStr">
+        <is>
+          <t>Bistec</t>
+        </is>
+      </c>
+      <c r="D280" s="68" t="inlineStr">
+        <is>
+          <t>Miscelánea LC La Cruz</t>
+        </is>
+      </c>
+      <c r="E280" s="69" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F280" s="70" t="n">
+        <v>285</v>
+      </c>
+      <c r="G280" s="23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H280" s="23" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I280" s="55" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Getnet **3982 · Aut 354977</t>
+        </is>
+      </c>
     </row>
     <row r="281">
-      <c r="B281" s="64" t="n"/>
-      <c r="C281" s="65" t="n"/>
-      <c r="D281" s="66" t="n"/>
-      <c r="E281" s="65" t="n"/>
-      <c r="F281" s="67" t="n"/>
-      <c r="G281" s="14" t="n"/>
-      <c r="H281" s="14" t="n"/>
-      <c r="I281" s="43" t="n"/>
+      <c r="B281" s="64" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C281" s="65" t="inlineStr">
+        <is>
+          <t>Tortillas Blancas</t>
+        </is>
+      </c>
+      <c r="D281" s="66" t="inlineStr">
+        <is>
+          <t>Local purchase</t>
+        </is>
+      </c>
+      <c r="E281" s="65" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F281" s="67" t="n">
+        <v>52</v>
+      </c>
+      <c r="G281" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H281" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I281" s="43" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>No receipt</t>
+        </is>
+      </c>
     </row>
     <row r="282">
-      <c r="B282" s="64" t="n"/>
-      <c r="C282" s="69" t="n"/>
-      <c r="D282" s="68" t="n"/>
-      <c r="E282" s="69" t="n"/>
-      <c r="F282" s="70" t="n"/>
-      <c r="G282" s="23" t="n"/>
-      <c r="H282" s="23" t="n"/>
-      <c r="I282" s="55" t="n"/>
+      <c r="B282" s="64" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C282" s="69" t="inlineStr">
+        <is>
+          <t>Leche Descremada, Jumex (2), Coca-Cola, CC Sin Azúcar, Crema (6 art.)</t>
+        </is>
+      </c>
+      <c r="D282" s="68" t="inlineStr">
+        <is>
+          <t>Sam’s Club</t>
+        </is>
+      </c>
+      <c r="E282" s="69" t="inlineStr">
+        <is>
+          <t>Supermarket / General</t>
+        </is>
+      </c>
+      <c r="F282" s="70" t="n">
+        <v>1386</v>
+      </c>
+      <c r="G282" s="23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H282" s="23" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I282" s="55" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Debit MC **82 · Aut 135301 · 12:46</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="B283" s="64" t="n"/>
@@ -38286,7 +38473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O209"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="30" customWidth="1" style="274" min="1" max="1"/>
@@ -39083,156 +39270,6 @@
       <c r="H59" s="93" t="n"/>
       <c r="I59" s="93" t="n"/>
     </row>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
updated additional Capital investment expenses
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -1169,7 +1169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="393">
+  <cellXfs count="397">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -2165,6 +2165,18 @@
     <xf numFmtId="4" fontId="88" fillId="19" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="174" fontId="73" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="73" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="74" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2629,7 +2641,7 @@
     <row r="2" ht="24" customHeight="1" s="274">
       <c r="B2" s="276" t="inlineStr">
         <is>
-          <t>Last updated: 10 Jun 2026  |  Capital, Acquisition, Pre-Opening &amp; Renovation CapEx</t>
+          <t>Last updated: 17 Jun 2026  |  Capital, Acquisition, Pre-Opening &amp; Renovation CapEx</t>
         </is>
       </c>
     </row>
@@ -2830,7 +2842,7 @@
       </c>
       <c r="F13" s="160" t="inlineStr">
         <is>
-          <t>⚠️ PARTIALLY PAID — $134,500 remaining</t>
+          <t>⚠️ PARTIALLY PAID — $118,970 remaining</t>
         </is>
       </c>
       <c r="G13" s="160" t="inlineStr">
@@ -3097,7 +3109,7 @@
       </c>
       <c r="C23" s="172" t="n"/>
       <c r="D23" s="180">
-        <f>D13-SUM(D14:D22)</f>
+        <f>D13-SUM(D14:D22)-D24</f>
         <v/>
       </c>
       <c r="E23" s="172" t="inlineStr">
@@ -3112,11 +3124,38 @@
       </c>
       <c r="G23" s="172" t="inlineStr">
         <is>
-          <t>$390,000 − $255,500 paid = $134,500 remaining</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="25.95" customHeight="1" s="274"/>
+          <t>$390,000 − $255,500 paid − $15,530 electricity offset = $118,970 remaining</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="25.95" customHeight="1" s="274">
+      <c r="B24" s="212" t="inlineStr">
+        <is>
+          <t>Electricity Bill (Mar–May CFE) — paid by Lohith for Previous Owners</t>
+        </is>
+      </c>
+      <c r="C24" s="393" t="n">
+        <v>46190</v>
+      </c>
+      <c r="D24" s="214" t="n">
+        <v>15530</v>
+      </c>
+      <c r="E24" s="213" t="inlineStr">
+        <is>
+          <t>Lohith Reddy</t>
+        </is>
+      </c>
+      <c r="F24" s="213" t="inlineStr">
+        <is>
+          <t>✅ OFFSET vs balance</t>
+        </is>
+      </c>
+      <c r="G24" s="212" t="inlineStr">
+        <is>
+          <t>Prev owners’ liability (pre-handover). Deducted from acquisition balance owed to them.</t>
+        </is>
+      </c>
+    </row>
     <row r="25" ht="22.05" customHeight="1" s="274">
       <c r="B25" s="173" t="inlineStr">
         <is>
@@ -3647,12 +3686,32 @@
       </c>
     </row>
     <row r="50" ht="22.05" customHeight="1" s="274">
-      <c r="B50" s="159" t="n"/>
-      <c r="C50" s="184" t="n"/>
-      <c r="D50" s="184" t="n"/>
-      <c r="E50" s="184" t="n"/>
-      <c r="F50" s="184" t="n"/>
-      <c r="G50" s="282" t="n"/>
+      <c r="B50" s="394" t="inlineStr">
+        <is>
+          <t>Alejandra — License Costs</t>
+        </is>
+      </c>
+      <c r="C50" s="393" t="n">
+        <v>46190</v>
+      </c>
+      <c r="D50" s="214" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E50" s="213" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="F50" s="213" t="inlineStr">
+        <is>
+          <t>Legal / License</t>
+        </is>
+      </c>
+      <c r="G50" s="212" t="inlineStr">
+        <is>
+          <t>License costs — paid by Lohith 17 Jun</t>
+        </is>
+      </c>
       <c r="H50" s="278" t="n"/>
     </row>
     <row r="51" ht="19.95" customHeight="1" s="274">
@@ -3934,12 +3993,32 @@
       </c>
     </row>
     <row r="66" ht="19.95" customHeight="1" s="274">
-      <c r="B66" s="159" t="n"/>
-      <c r="C66" s="159" t="n"/>
-      <c r="D66" s="185" t="n"/>
-      <c r="E66" s="159" t="n"/>
-      <c r="F66" s="159" t="n"/>
-      <c r="G66" s="159" t="n"/>
+      <c r="B66" s="394" t="inlineStr">
+        <is>
+          <t>Letrero 3-D Retroiluminado (illuminated sign)</t>
+        </is>
+      </c>
+      <c r="C66" s="395" t="n">
+        <v>46190</v>
+      </c>
+      <c r="D66" s="396" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E66" s="394" t="inlineStr">
+        <is>
+          <t>POPA Publicidad</t>
+        </is>
+      </c>
+      <c r="F66" s="394" t="inlineStr">
+        <is>
+          <t>Branding / Signage</t>
+        </is>
+      </c>
+      <c r="G66" s="394" t="inlineStr">
+        <is>
+          <t>3D backlit sign + "CAFE RESTAURANT &amp; BAR" letters — paid by Shashirekha · Cotización A0626-560</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="19.95" customHeight="1" s="274">
       <c r="B67" s="212" t="n"/>
@@ -4621,10 +4700,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B24:H24"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B11:H11"/>
   </mergeCells>
@@ -27178,14 +27256,47 @@
       </c>
     </row>
     <row r="283">
-      <c r="B283" s="64" t="n"/>
-      <c r="C283" s="65" t="n"/>
-      <c r="D283" s="66" t="n"/>
-      <c r="E283" s="65" t="n"/>
-      <c r="F283" s="67" t="n"/>
-      <c r="G283" s="14" t="n"/>
-      <c r="H283" s="14" t="n"/>
-      <c r="I283" s="43" t="n"/>
+      <c r="B283" s="64" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C283" s="65" t="inlineStr">
+        <is>
+          <t>Detergente Roma 2kg + Blanqueador Clorox 5.8L</t>
+        </is>
+      </c>
+      <c r="D283" s="66" t="inlineStr">
+        <is>
+          <t>Chedraui Paseo</t>
+        </is>
+      </c>
+      <c r="E283" s="65" t="inlineStr">
+        <is>
+          <t>Supplies / Other</t>
+        </is>
+      </c>
+      <c r="F283" s="67" t="n">
+        <v>157</v>
+      </c>
+      <c r="G283" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H283" s="14" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I283" s="43" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Débito **3982 · Aut 161026 · cleaning supplies</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="B284" s="64" t="n"/>
@@ -38479,7 +38590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O209"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="32" customWidth="1" style="274" min="1" max="1"/>
@@ -39276,156 +39387,6 @@
       <c r="H59" s="93" t="n"/>
       <c r="I59" s="93" t="n"/>
     </row>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
Updated few other expenses
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -25,7 +25,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ ddd"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
@@ -38,6 +38,7 @@
     <numFmt numFmtId="173" formatCode="#,##0;\-#,##0;\-"/>
     <numFmt numFmtId="174" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="175" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="98">
     <font>
@@ -976,7 +977,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -1283,11 +1284,15 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19"/>
   </cellStyleXfs>
-  <cellXfs count="382">
+  <cellXfs count="393">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -2272,6 +2277,37 @@
     <xf numFmtId="3" fontId="94" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="176" fontId="51" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="95" fillId="57" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="37" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="19" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="41" fillId="19" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="42" fillId="17" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="43" fillId="19" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="44" fillId="19" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="19" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9518,17 +9554,45 @@
       <c r="Q41" s="56" t="n"/>
     </row>
     <row r="42" ht="16.5" customHeight="1" s="278">
-      <c r="B42" s="34" t="n"/>
-      <c r="C42" s="35" t="n"/>
-      <c r="D42" s="36" t="n"/>
-      <c r="E42" s="37" t="n"/>
-      <c r="F42" s="38" t="n"/>
-      <c r="G42" s="39" t="n"/>
-      <c r="H42" s="40" t="n"/>
-      <c r="I42" s="41" t="n"/>
-      <c r="J42" s="42" t="n"/>
-      <c r="K42" s="43" t="n"/>
-      <c r="L42" s="9" t="n"/>
+      <c r="B42" s="385" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C42" s="386" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="D42" s="387" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="38">
+        <f>IFERROR(D42+E42+G42,0)</f>
+        <v/>
+      </c>
+      <c r="G42" s="388" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="389">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B42,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B42+1))</f>
+        <v/>
+      </c>
+      <c r="I42" s="390">
+        <f>IFERROR(F42-H42,0)</f>
+        <v/>
+      </c>
+      <c r="J42" s="391">
+        <f>IFERROR(I42/F42,0)</f>
+        <v/>
+      </c>
+      <c r="K42" s="251" t="n"/>
+      <c r="L42" s="392" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
       <c r="M42" s="12" t="n"/>
       <c r="N42" s="44" t="n"/>
       <c r="O42" s="45" t="n"/>
@@ -15477,8 +15541,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -28140,184 +28204,762 @@
       </c>
     </row>
     <row r="306">
-      <c r="B306" s="64" t="n"/>
-      <c r="C306" s="69" t="n"/>
-      <c r="D306" s="68" t="n"/>
-      <c r="E306" s="69" t="n"/>
-      <c r="F306" s="70" t="n"/>
-      <c r="G306" s="23" t="n"/>
-      <c r="H306" s="23" t="n"/>
-      <c r="I306" s="55" t="n"/>
+      <c r="B306" s="382" t="n">
+        <v>46176</v>
+      </c>
+      <c r="C306" s="252" t="inlineStr">
+        <is>
+          <t>Cuchara de Moka 6pcs 10.5cm (x2)</t>
+        </is>
+      </c>
+      <c r="D306" s="253" t="inlineStr">
+        <is>
+          <t>Small China</t>
+        </is>
+      </c>
+      <c r="E306" s="252" t="inlineStr">
+        <is>
+          <t>Kitchen Supplies</t>
+        </is>
+      </c>
+      <c r="F306" s="70" t="n">
+        <v>178</v>
+      </c>
+      <c r="G306" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H306" s="254" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I306" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J306" s="383" t="inlineStr">
+        <is>
+          <t>Tarjeta crédito · serial D2606031530065 (back-dated 3 Jun)</t>
+        </is>
+      </c>
     </row>
     <row r="307">
-      <c r="B307" s="64" t="n"/>
-      <c r="C307" s="65" t="n"/>
-      <c r="D307" s="66" t="n"/>
-      <c r="E307" s="65" t="n"/>
-      <c r="F307" s="67" t="n"/>
-      <c r="G307" s="14" t="n"/>
-      <c r="H307" s="14" t="n"/>
-      <c r="I307" s="43" t="n"/>
+      <c r="B307" s="382" t="n">
+        <v>46193</v>
+      </c>
+      <c r="C307" s="248" t="inlineStr">
+        <is>
+          <t>Topo Chico (2 packs)</t>
+        </is>
+      </c>
+      <c r="D307" s="249" t="inlineStr">
+        <is>
+          <t>Sam's Club</t>
+        </is>
+      </c>
+      <c r="E307" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Beverages</t>
+        </is>
+      </c>
+      <c r="F307" s="67" t="n">
+        <v>464</v>
+      </c>
+      <c r="G307" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H307" s="250" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I307" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J307" s="383" t="inlineStr">
+        <is>
+          <t>No receipt</t>
+        </is>
+      </c>
     </row>
     <row r="308">
-      <c r="B308" s="64" t="n"/>
-      <c r="C308" s="69" t="n"/>
-      <c r="D308" s="68" t="n"/>
-      <c r="E308" s="69" t="n"/>
-      <c r="F308" s="70" t="n"/>
-      <c r="G308" s="23" t="n"/>
-      <c r="H308" s="23" t="n"/>
-      <c r="I308" s="55" t="n"/>
+      <c r="B308" s="382" t="n">
+        <v>46192</v>
+      </c>
+      <c r="C308" s="252" t="inlineStr">
+        <is>
+          <t>Soft Restaurant — POS app subscription</t>
+        </is>
+      </c>
+      <c r="D308" s="253" t="inlineStr">
+        <is>
+          <t>Soft Restaurant</t>
+        </is>
+      </c>
+      <c r="E308" s="252" t="inlineStr">
+        <is>
+          <t>Software / Subscription</t>
+        </is>
+      </c>
+      <c r="F308" s="70" t="n">
+        <v>810</v>
+      </c>
+      <c r="G308" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H308" s="254" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I308" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J308" s="383" t="inlineStr">
+        <is>
+          <t>No receipt · POS software subscription</t>
+        </is>
+      </c>
     </row>
     <row r="309">
-      <c r="B309" s="64" t="n"/>
-      <c r="C309" s="65" t="n"/>
-      <c r="D309" s="66" t="n"/>
-      <c r="E309" s="65" t="n"/>
-      <c r="F309" s="67" t="n"/>
-      <c r="G309" s="14" t="n"/>
-      <c r="H309" s="14" t="n"/>
-      <c r="I309" s="43" t="n"/>
+      <c r="B309" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C309" s="248" t="inlineStr">
+        <is>
+          <t>Morrón surtido, espinaca, betabel</t>
+        </is>
+      </c>
+      <c r="D309" s="249" t="inlineStr">
+        <is>
+          <t>Verduras Selectas Oscar</t>
+        </is>
+      </c>
+      <c r="E309" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F309" s="67" t="n">
+        <v>84</v>
+      </c>
+      <c r="G309" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H309" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I309" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J309" s="383" t="inlineStr">
+        <is>
+          <t>Mercado de Abastos</t>
+        </is>
+      </c>
     </row>
     <row r="310">
-      <c r="B310" s="64" t="n"/>
-      <c r="C310" s="69" t="n"/>
-      <c r="D310" s="68" t="n"/>
-      <c r="E310" s="69" t="n"/>
-      <c r="F310" s="70" t="n"/>
-      <c r="G310" s="23" t="n"/>
-      <c r="H310" s="23" t="n"/>
-      <c r="I310" s="55" t="n"/>
+      <c r="B310" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C310" s="252" t="inlineStr">
+        <is>
+          <t>Champiñón 1.02kg + Manzana Mexicana 1.13kg</t>
+        </is>
+      </c>
+      <c r="D310" s="253" t="inlineStr">
+        <is>
+          <t>Mercado de Abastos</t>
+        </is>
+      </c>
+      <c r="E310" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F310" s="70" t="n">
+        <v>153.62</v>
+      </c>
+      <c r="G310" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H310" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I310" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J310" s="383" t="inlineStr">
+        <is>
+          <t>Ticket 26351 (incl. apple)</t>
+        </is>
+      </c>
     </row>
     <row r="311">
-      <c r="B311" s="64" t="n"/>
-      <c r="C311" s="65" t="n"/>
-      <c r="D311" s="66" t="n"/>
-      <c r="E311" s="65" t="n"/>
-      <c r="F311" s="67" t="n"/>
-      <c r="G311" s="14" t="n"/>
-      <c r="H311" s="14" t="n"/>
-      <c r="I311" s="43" t="n"/>
+      <c r="B311" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C311" s="248" t="inlineStr">
+        <is>
+          <t>Huevo (2 conos)</t>
+        </is>
+      </c>
+      <c r="D311" s="249" t="inlineStr">
+        <is>
+          <t>Jaime (Mercado Abastos)</t>
+        </is>
+      </c>
+      <c r="E311" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Eggs</t>
+        </is>
+      </c>
+      <c r="F311" s="67" t="n">
+        <v>102</v>
+      </c>
+      <c r="G311" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H311" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I311" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J311" s="383" t="inlineStr"/>
     </row>
     <row r="312">
-      <c r="B312" s="64" t="n"/>
-      <c r="C312" s="69" t="n"/>
-      <c r="D312" s="68" t="n"/>
-      <c r="E312" s="69" t="n"/>
-      <c r="F312" s="70" t="n"/>
-      <c r="G312" s="23" t="n"/>
-      <c r="H312" s="23" t="n"/>
-      <c r="I312" s="55" t="n"/>
+      <c r="B312" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C312" s="252" t="inlineStr">
+        <is>
+          <t>Zanahoria, jalapeño, serrano, cebolla</t>
+        </is>
+      </c>
+      <c r="D312" s="253" t="inlineStr">
+        <is>
+          <t>Mi Joven</t>
+        </is>
+      </c>
+      <c r="E312" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F312" s="70" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="G312" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H312" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I312" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J312" s="383" t="inlineStr">
+        <is>
+          <t>Folio 19465</t>
+        </is>
+      </c>
     </row>
     <row r="313">
-      <c r="B313" s="64" t="n"/>
-      <c r="C313" s="65" t="n"/>
-      <c r="D313" s="66" t="n"/>
-      <c r="E313" s="65" t="n"/>
-      <c r="F313" s="67" t="n"/>
-      <c r="G313" s="14" t="n"/>
-      <c r="H313" s="14" t="n"/>
-      <c r="I313" s="43" t="n"/>
+      <c r="B313" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C313" s="248" t="inlineStr">
+        <is>
+          <t>Calabaza 1.7kg</t>
+        </is>
+      </c>
+      <c r="D313" s="249" t="inlineStr">
+        <is>
+          <t>Mi Joven</t>
+        </is>
+      </c>
+      <c r="E313" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F313" s="67" t="n">
+        <v>34</v>
+      </c>
+      <c r="G313" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H313" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I313" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J313" s="383" t="inlineStr">
+        <is>
+          <t>Folio 19466</t>
+        </is>
+      </c>
     </row>
     <row r="314">
-      <c r="B314" s="64" t="n"/>
-      <c r="C314" s="69" t="n"/>
-      <c r="D314" s="68" t="n"/>
-      <c r="E314" s="69" t="n"/>
-      <c r="F314" s="70" t="n"/>
-      <c r="G314" s="23" t="n"/>
-      <c r="H314" s="23" t="n"/>
-      <c r="I314" s="55" t="n"/>
+      <c r="B314" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C314" s="252" t="inlineStr">
+        <is>
+          <t>Tomate, limón, pepino, jícama</t>
+        </is>
+      </c>
+      <c r="D314" s="253" t="inlineStr">
+        <is>
+          <t>Mercado de Abastos</t>
+        </is>
+      </c>
+      <c r="E314" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F314" s="70" t="n">
+        <v>240</v>
+      </c>
+      <c r="G314" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H314" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I314" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J314" s="383" t="inlineStr">
+        <is>
+          <t>Handwritten note</t>
+        </is>
+      </c>
     </row>
     <row r="315">
-      <c r="B315" s="64" t="n"/>
-      <c r="C315" s="65" t="n"/>
-      <c r="D315" s="66" t="n"/>
-      <c r="E315" s="65" t="n"/>
-      <c r="F315" s="67" t="n"/>
-      <c r="G315" s="14" t="n"/>
-      <c r="H315" s="14" t="n"/>
-      <c r="I315" s="43" t="n"/>
+      <c r="B315" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C315" s="248" t="inlineStr">
+        <is>
+          <t>Jitomate 7kg</t>
+        </is>
+      </c>
+      <c r="D315" s="249" t="inlineStr">
+        <is>
+          <t>Frutas Finas Ana Pao</t>
+        </is>
+      </c>
+      <c r="E315" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F315" s="67" t="n">
+        <v>105</v>
+      </c>
+      <c r="G315" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H315" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I315" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J315" s="383" t="inlineStr"/>
     </row>
     <row r="316">
-      <c r="B316" s="64" t="n"/>
-      <c r="C316" s="69" t="n"/>
-      <c r="D316" s="68" t="n"/>
-      <c r="E316" s="69" t="n"/>
-      <c r="F316" s="70" t="n"/>
-      <c r="G316" s="23" t="n"/>
-      <c r="H316" s="23" t="n"/>
-      <c r="I316" s="55" t="n"/>
+      <c r="B316" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C316" s="252" t="inlineStr">
+        <is>
+          <t>Sandía, papaya, plátano, melón</t>
+        </is>
+      </c>
+      <c r="D316" s="253" t="inlineStr">
+        <is>
+          <t>Mercado de Abastos</t>
+        </is>
+      </c>
+      <c r="E316" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Fruit</t>
+        </is>
+      </c>
+      <c r="F316" s="70" t="n">
+        <v>208</v>
+      </c>
+      <c r="G316" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H316" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I316" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J316" s="383" t="inlineStr">
+        <is>
+          <t>Handwritten note</t>
+        </is>
+      </c>
     </row>
     <row r="317">
-      <c r="B317" s="64" t="n"/>
-      <c r="C317" s="65" t="n"/>
-      <c r="D317" s="66" t="n"/>
-      <c r="E317" s="65" t="n"/>
-      <c r="F317" s="67" t="n"/>
-      <c r="G317" s="14" t="n"/>
-      <c r="H317" s="14" t="n"/>
-      <c r="I317" s="43" t="n"/>
+      <c r="B317" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C317" s="248" t="inlineStr">
+        <is>
+          <t>Papa (3 x $35)</t>
+        </is>
+      </c>
+      <c r="D317" s="249" t="inlineStr">
+        <is>
+          <t>Papas San Miguel</t>
+        </is>
+      </c>
+      <c r="E317" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F317" s="67" t="n">
+        <v>105</v>
+      </c>
+      <c r="G317" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H317" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I317" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J317" s="383" t="inlineStr"/>
     </row>
     <row r="318">
-      <c r="B318" s="64" t="n"/>
-      <c r="C318" s="69" t="n"/>
-      <c r="D318" s="68" t="n"/>
-      <c r="E318" s="69" t="n"/>
-      <c r="F318" s="70" t="n"/>
-      <c r="G318" s="23" t="n"/>
-      <c r="H318" s="23" t="n"/>
-      <c r="I318" s="55" t="n"/>
+      <c r="B318" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C318" s="252" t="inlineStr">
+        <is>
+          <t>Aguacate Hass + habanero</t>
+        </is>
+      </c>
+      <c r="D318" s="253" t="inlineStr">
+        <is>
+          <t>Rey Tacamba</t>
+        </is>
+      </c>
+      <c r="E318" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F318" s="70" t="n">
+        <v>214</v>
+      </c>
+      <c r="G318" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H318" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I318" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J318" s="383" t="inlineStr">
+        <is>
+          <t>Hass $94 + habanero $120</t>
+        </is>
+      </c>
     </row>
     <row r="319">
-      <c r="B319" s="64" t="n"/>
-      <c r="C319" s="65" t="n"/>
-      <c r="D319" s="66" t="n"/>
-      <c r="E319" s="65" t="n"/>
-      <c r="F319" s="67" t="n"/>
-      <c r="G319" s="14" t="n"/>
-      <c r="H319" s="14" t="n"/>
-      <c r="I319" s="43" t="n"/>
+      <c r="B319" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C319" s="248" t="inlineStr">
+        <is>
+          <t>Chicharrón (1 hoja)</t>
+        </is>
+      </c>
+      <c r="D319" s="249" t="inlineStr">
+        <is>
+          <t>Chicharronería San Nicolás</t>
+        </is>
+      </c>
+      <c r="E319" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F319" s="67" t="n">
+        <v>89</v>
+      </c>
+      <c r="G319" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H319" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I319" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J319" s="383" t="inlineStr">
+        <is>
+          <t>Corrected to \ per Reddy (was read as 899)</t>
+        </is>
+      </c>
     </row>
     <row r="320">
-      <c r="B320" s="64" t="n"/>
-      <c r="C320" s="69" t="n"/>
-      <c r="D320" s="68" t="n"/>
-      <c r="E320" s="69" t="n"/>
-      <c r="F320" s="70" t="n"/>
-      <c r="G320" s="23" t="n"/>
-      <c r="H320" s="23" t="n"/>
-      <c r="I320" s="55" t="n"/>
+      <c r="B320" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C320" s="252" t="inlineStr">
+        <is>
+          <t>Vasos, tapas, cucharas, biocup vaso papel</t>
+        </is>
+      </c>
+      <c r="D320" s="253" t="inlineStr">
+        <is>
+          <t>MPPD - Materias Primas Plasticos</t>
+        </is>
+      </c>
+      <c r="E320" s="252" t="inlineStr">
+        <is>
+          <t>Packaging / Disposables</t>
+        </is>
+      </c>
+      <c r="F320" s="70" t="n">
+        <v>295.73</v>
+      </c>
+      <c r="G320" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H320" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I320" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J320" s="383" t="inlineStr">
+        <is>
+          <t>Folio 381088</t>
+        </is>
+      </c>
     </row>
     <row r="321">
-      <c r="B321" s="64" t="n"/>
-      <c r="C321" s="65" t="n"/>
-      <c r="D321" s="66" t="n"/>
-      <c r="E321" s="65" t="n"/>
-      <c r="F321" s="67" t="n"/>
-      <c r="G321" s="14" t="n"/>
-      <c r="H321" s="14" t="n"/>
-      <c r="I321" s="43" t="n"/>
+      <c r="B321" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C321" s="248" t="inlineStr">
+        <is>
+          <t>Cilantro, hierbabuena, lechuga italiana</t>
+        </is>
+      </c>
+      <c r="D321" s="249" t="inlineStr">
+        <is>
+          <t>Hnos. Labra's</t>
+        </is>
+      </c>
+      <c r="E321" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F321" s="67" t="n">
+        <v>215</v>
+      </c>
+      <c r="G321" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H321" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I321" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J321" s="383" t="inlineStr"/>
     </row>
     <row r="322">
-      <c r="B322" s="64" t="n"/>
-      <c r="C322" s="69" t="n"/>
-      <c r="D322" s="68" t="n"/>
-      <c r="E322" s="69" t="n"/>
-      <c r="F322" s="70" t="n"/>
-      <c r="G322" s="23" t="n"/>
-      <c r="H322" s="23" t="n"/>
-      <c r="I322" s="55" t="n"/>
+      <c r="B322" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C322" s="252" t="inlineStr">
+        <is>
+          <t>Pens (office/stationery)</t>
+        </is>
+      </c>
+      <c r="D322" s="253" t="inlineStr">
+        <is>
+          <t>Local purchase</t>
+        </is>
+      </c>
+      <c r="E322" s="252" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F322" s="70" t="n">
+        <v>30</v>
+      </c>
+      <c r="G322" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H322" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I322" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J322" s="383" t="inlineStr">
+        <is>
+          <t>No receipt</t>
+        </is>
+      </c>
     </row>
     <row r="323">
-      <c r="B323" s="64" t="n"/>
-      <c r="C323" s="65" t="n"/>
-      <c r="D323" s="66" t="n"/>
-      <c r="E323" s="65" t="n"/>
-      <c r="F323" s="67" t="n"/>
-      <c r="G323" s="14" t="n"/>
-      <c r="H323" s="14" t="n"/>
-      <c r="I323" s="43" t="n"/>
+      <c r="B323" s="382" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C323" s="248" t="inlineStr">
+        <is>
+          <t>Restaurant Command booklet (comandas)</t>
+        </is>
+      </c>
+      <c r="D323" s="249" t="inlineStr">
+        <is>
+          <t>Local purchase</t>
+        </is>
+      </c>
+      <c r="E323" s="248" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F323" s="67" t="n">
+        <v>59</v>
+      </c>
+      <c r="G323" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H323" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I323" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J323" s="383" t="inlineStr">
+        <is>
+          <t>No receipt — order pads</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="B324" s="64" t="n"/>
@@ -39855,7 +40497,7 @@
     <row r="21">
       <c r="A21" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Pantry</t>
+          <t>Ingredients - Beverages</t>
         </is>
       </c>
       <c r="B21" s="378">
@@ -39879,7 +40521,7 @@
     <row r="22">
       <c r="A22" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Beverages</t>
+          <t>Ingredients - Pantry</t>
         </is>
       </c>
       <c r="B22" s="378">
@@ -40071,7 +40713,7 @@
     <row r="30">
       <c r="A30" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Other</t>
+          <t>Software / Subscription</t>
         </is>
       </c>
       <c r="B30" s="378">
@@ -40095,7 +40737,7 @@
     <row r="31">
       <c r="A31" s="380" t="inlineStr">
         <is>
-          <t>Staff - Advance</t>
+          <t>Ingredients - Other</t>
         </is>
       </c>
       <c r="B31" s="378">
@@ -40119,7 +40761,7 @@
     <row r="32">
       <c r="A32" s="380" t="inlineStr">
         <is>
-          <t>Utilities / Internet</t>
+          <t>Staff - Advance</t>
         </is>
       </c>
       <c r="B32" s="378">
@@ -40143,7 +40785,7 @@
     <row r="33">
       <c r="A33" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Desserts</t>
+          <t>Utilities / Internet</t>
         </is>
       </c>
       <c r="B33" s="378">
@@ -40167,7 +40809,7 @@
     <row r="34">
       <c r="A34" s="380" t="inlineStr">
         <is>
-          <t>Staff - Propinas</t>
+          <t>Packaging / Disposables</t>
         </is>
       </c>
       <c r="B34" s="378">
@@ -40191,7 +40833,7 @@
     <row r="35">
       <c r="A35" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Produce</t>
+          <t>Ingredients - Desserts</t>
         </is>
       </c>
       <c r="B35" s="378">
@@ -40213,17 +40855,17 @@
       <c r="L35" s="374" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="377" t="inlineStr">
-        <is>
-          <t>TOTAL EXPENSES</t>
-        </is>
-      </c>
-      <c r="B36" s="379">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
-        <v/>
-      </c>
-      <c r="C36" s="379">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+      <c r="A36" s="380" t="inlineStr">
+        <is>
+          <t>Kitchen Supplies</t>
+        </is>
+      </c>
+      <c r="B36" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A36,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C36" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A36,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D36" s="374" t="n"/>
@@ -40237,17 +40879,17 @@
       <c r="L36" s="374" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="377" t="inlineStr">
-        <is>
-          <t>NET PROFIT / LOSS</t>
-        </is>
-      </c>
-      <c r="B37" s="379">
-        <f>B4-B36</f>
-        <v/>
-      </c>
-      <c r="C37" s="379">
-        <f>C4-C36</f>
+      <c r="A37" s="380" t="inlineStr">
+        <is>
+          <t>Staff - Propinas</t>
+        </is>
+      </c>
+      <c r="B37" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A37,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C37" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A37,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D37" s="374" t="n"/>
@@ -40261,9 +40903,19 @@
       <c r="L37" s="374" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="374" t="n"/>
-      <c r="B38" s="374" t="n"/>
-      <c r="C38" s="374" t="n"/>
+      <c r="A38" s="380" t="inlineStr">
+        <is>
+          <t>Ingredients - Eggs</t>
+        </is>
+      </c>
+      <c r="B38" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A38,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C38" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A38,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <v/>
+      </c>
       <c r="D38" s="374" t="n"/>
       <c r="E38" s="374" t="n"/>
       <c r="F38" s="374" t="n"/>
@@ -40275,9 +40927,19 @@
       <c r="L38" s="374" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="374" t="n"/>
-      <c r="B39" s="374" t="n"/>
-      <c r="C39" s="374" t="n"/>
+      <c r="A39" s="380" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="B39" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A39,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C39" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A39,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <v/>
+      </c>
       <c r="D39" s="374" t="n"/>
       <c r="E39" s="374" t="n"/>
       <c r="F39" s="374" t="n"/>
@@ -40289,9 +40951,19 @@
       <c r="L39" s="374" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="374" t="n"/>
-      <c r="B40" s="374" t="n"/>
-      <c r="C40" s="374" t="n"/>
+      <c r="A40" s="380" t="inlineStr">
+        <is>
+          <t>Ingredients - Produce</t>
+        </is>
+      </c>
+      <c r="B40" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A40,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C40" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A40,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <v/>
+      </c>
       <c r="D40" s="374" t="n"/>
       <c r="E40" s="374" t="n"/>
       <c r="F40" s="374" t="n"/>
@@ -40303,9 +40975,19 @@
       <c r="L40" s="374" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="374" t="n"/>
-      <c r="B41" s="374" t="n"/>
-      <c r="C41" s="374" t="n"/>
+      <c r="A41" s="377" t="inlineStr">
+        <is>
+          <t>TOTAL EXPENSES</t>
+        </is>
+      </c>
+      <c r="B41" s="379">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C41" s="379">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <v/>
+      </c>
       <c r="D41" s="374" t="n"/>
       <c r="E41" s="374" t="n"/>
       <c r="F41" s="374" t="n"/>
@@ -40317,9 +40999,19 @@
       <c r="L41" s="374" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="374" t="n"/>
-      <c r="B42" s="374" t="n"/>
-      <c r="C42" s="374" t="n"/>
+      <c r="A42" s="377" t="inlineStr">
+        <is>
+          <t>NET PROFIT / LOSS</t>
+        </is>
+      </c>
+      <c r="B42" s="379">
+        <f>B4-B41</f>
+        <v/>
+      </c>
+      <c r="C42" s="379">
+        <f>C4-C41</f>
+        <v/>
+      </c>
       <c r="D42" s="374" t="n"/>
       <c r="E42" s="374" t="n"/>
       <c r="F42" s="374" t="n"/>

</xml_diff>

<commit_message>
updated this week details
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -10623,7 +10623,7 @@
         <v>3702</v>
       </c>
       <c r="E54" s="37" t="n">
-        <v>2265</v>
+        <v>2375</v>
       </c>
       <c r="F54" s="38">
         <f>IFERROR(D54+E54+G54,0)</f>
@@ -10644,7 +10644,11 @@
         <f>IFERROR(I54/F54,0)</f>
         <v/>
       </c>
-      <c r="K54" s="251" t="n"/>
+      <c r="K54" s="251" t="inlineStr">
+        <is>
+          <t>incl +$110 additional cash income (added 04-Jul)</t>
+        </is>
+      </c>
       <c r="L54" s="392" t="inlineStr">
         <is>
           <t>Cierre via loka.py</t>
@@ -10661,22 +10665,54 @@
       </c>
     </row>
     <row r="55" ht="16.5" customHeight="1" s="278">
-      <c r="B55" s="34" t="n"/>
-      <c r="C55" s="47" t="n"/>
-      <c r="D55" s="48" t="n"/>
-      <c r="E55" s="49" t="n"/>
-      <c r="F55" s="50" t="n"/>
-      <c r="G55" s="51" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="53" t="n"/>
-      <c r="J55" s="54" t="n"/>
-      <c r="K55" s="55" t="n"/>
-      <c r="L55" s="18" t="n"/>
+      <c r="B55" s="385" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C55" s="256" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D55" s="257" t="n">
+        <v>1739</v>
+      </c>
+      <c r="E55" s="49" t="n">
+        <v>895</v>
+      </c>
+      <c r="F55" s="50">
+        <f>IFERROR(D55+E55+G55,0)</f>
+        <v/>
+      </c>
+      <c r="G55" s="258" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="259">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B55,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B55+1))</f>
+        <v/>
+      </c>
+      <c r="I55" s="260">
+        <f>IFERROR(F55-H55,0)</f>
+        <v/>
+      </c>
+      <c r="J55" s="261">
+        <f>IFERROR(I55/F55,0)</f>
+        <v/>
+      </c>
+      <c r="K55" s="255" t="n"/>
+      <c r="L55" s="262" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
       <c r="M55" s="21" t="n"/>
       <c r="N55" s="56" t="n"/>
       <c r="O55" s="57" t="n"/>
       <c r="P55" s="58" t="n"/>
       <c r="Q55" s="56" t="n"/>
+      <c r="R55" s="410">
+        <f>IFERROR(D55*$T$7,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="16.5" customHeight="1" s="278">
       <c r="B56" s="34" t="n"/>
@@ -16386,9 +16422,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -33806,164 +33842,692 @@
       </c>
     </row>
     <row r="417">
-      <c r="B417" s="64" t="n"/>
-      <c r="C417" s="65" t="n"/>
-      <c r="D417" s="66" t="n"/>
-      <c r="E417" s="65" t="n"/>
-      <c r="F417" s="67" t="n"/>
-      <c r="G417" s="14" t="n"/>
-      <c r="H417" s="14" t="n"/>
-      <c r="I417" s="43" t="n"/>
+      <c r="B417" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C417" s="248" t="inlineStr">
+        <is>
+          <t>Zanahoria 3kg, Limon 3kg, Cebolla 3kg</t>
+        </is>
+      </c>
+      <c r="D417" s="249" t="inlineStr">
+        <is>
+          <t>Mi Joven</t>
+        </is>
+      </c>
+      <c r="E417" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F417" s="67" t="n">
+        <v>147</v>
+      </c>
+      <c r="G417" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H417" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I417" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J417" s="383" t="inlineStr">
+        <is>
+          <t>Mercado de Abastos folio 21212; efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="418">
-      <c r="B418" s="64" t="n"/>
-      <c r="C418" s="69" t="n"/>
-      <c r="D418" s="68" t="n"/>
-      <c r="E418" s="69" t="n"/>
-      <c r="F418" s="70" t="n"/>
-      <c r="G418" s="23" t="n"/>
-      <c r="H418" s="23" t="n"/>
-      <c r="I418" s="55" t="n"/>
+      <c r="B418" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C418" s="252" t="inlineStr">
+        <is>
+          <t>Papas 6 x $35</t>
+        </is>
+      </c>
+      <c r="D418" s="253" t="inlineStr">
+        <is>
+          <t>Papas San Miguel</t>
+        </is>
+      </c>
+      <c r="E418" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F418" s="70" t="n">
+        <v>210</v>
+      </c>
+      <c r="G418" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H418" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I418" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J418" s="383" t="inlineStr">
+        <is>
+          <t>6x35=210; efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="419">
-      <c r="B419" s="64" t="n"/>
-      <c r="C419" s="65" t="n"/>
-      <c r="D419" s="66" t="n"/>
-      <c r="E419" s="65" t="n"/>
-      <c r="F419" s="67" t="n"/>
-      <c r="G419" s="14" t="n"/>
-      <c r="H419" s="14" t="n"/>
-      <c r="I419" s="43" t="n"/>
+      <c r="B419" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C419" s="248" t="inlineStr">
+        <is>
+          <t>Verduras/hierbas mixtas (col, espinacas, hierbabuena, champinones, betabeles, lechugas, jengibre)</t>
+        </is>
+      </c>
+      <c r="D419" s="249" t="inlineStr">
+        <is>
+          <t>Hnos. Labra</t>
+        </is>
+      </c>
+      <c r="E419" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F419" s="67" t="n">
+        <v>339</v>
+      </c>
+      <c r="G419" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H419" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I419" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J419" s="383" t="inlineStr">
+        <is>
+          <t>Suma lineas=339; efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="420">
-      <c r="B420" s="64" t="n"/>
-      <c r="C420" s="69" t="n"/>
-      <c r="D420" s="68" t="n"/>
-      <c r="E420" s="69" t="n"/>
-      <c r="F420" s="70" t="n"/>
-      <c r="G420" s="23" t="n"/>
-      <c r="H420" s="23" t="n"/>
-      <c r="I420" s="55" t="n"/>
+      <c r="B420" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C420" s="252" t="inlineStr">
+        <is>
+          <t>Guayaba (1 primera)</t>
+        </is>
+      </c>
+      <c r="D420" s="253" t="inlineStr">
+        <is>
+          <t>Guayabas Aviles Hernandez</t>
+        </is>
+      </c>
+      <c r="E420" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Fruit</t>
+        </is>
+      </c>
+      <c r="F420" s="70" t="n">
+        <v>150</v>
+      </c>
+      <c r="G420" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H420" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I420" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J420" s="383" t="inlineStr">
+        <is>
+          <t>Total ~$150; efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="421">
-      <c r="B421" s="64" t="n"/>
-      <c r="C421" s="65" t="n"/>
-      <c r="D421" s="66" t="n"/>
-      <c r="E421" s="65" t="n"/>
-      <c r="F421" s="67" t="n"/>
-      <c r="G421" s="14" t="n"/>
-      <c r="H421" s="14" t="n"/>
-      <c r="I421" s="43" t="n"/>
+      <c r="B421" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C421" s="248" t="inlineStr">
+        <is>
+          <t>Pepino</t>
+        </is>
+      </c>
+      <c r="D421" s="249" t="inlineStr">
+        <is>
+          <t>Citricos Sanchez</t>
+        </is>
+      </c>
+      <c r="E421" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F421" s="67" t="n">
+        <v>49</v>
+      </c>
+      <c r="G421" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H421" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I421" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J421" s="383" t="inlineStr">
+        <is>
+          <t>Folio 7244; total $49 (detalle de linea poco legible)</t>
+        </is>
+      </c>
     </row>
     <row r="422">
-      <c r="B422" s="64" t="n"/>
-      <c r="C422" s="69" t="n"/>
-      <c r="D422" s="68" t="n"/>
-      <c r="E422" s="69" t="n"/>
-      <c r="F422" s="70" t="n"/>
-      <c r="G422" s="23" t="n"/>
-      <c r="H422" s="23" t="n"/>
-      <c r="I422" s="55" t="n"/>
+      <c r="B422" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C422" s="252" t="inlineStr">
+        <is>
+          <t>Cubiertos soperos desechables (tenedor/cuchara/cuchillo)</t>
+        </is>
+      </c>
+      <c r="D422" s="253" t="inlineStr">
+        <is>
+          <t>Guimar Polietilenos</t>
+        </is>
+      </c>
+      <c r="E422" s="252" t="inlineStr">
+        <is>
+          <t>Packaging/Disposables</t>
+        </is>
+      </c>
+      <c r="F422" s="70" t="n">
+        <v>139.8</v>
+      </c>
+      <c r="G422" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H422" s="254" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I422" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J422" s="383" t="inlineStr">
+        <is>
+          <t>Folio AK90544; tarjeta de credito</t>
+        </is>
+      </c>
     </row>
     <row r="423">
-      <c r="B423" s="64" t="n"/>
-      <c r="C423" s="65" t="n"/>
-      <c r="D423" s="66" t="n"/>
-      <c r="E423" s="65" t="n"/>
-      <c r="F423" s="67" t="n"/>
-      <c r="G423" s="14" t="n"/>
-      <c r="H423" s="14" t="n"/>
-      <c r="I423" s="43" t="n"/>
+      <c r="B423" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C423" s="248" t="inlineStr">
+        <is>
+          <t>Melon</t>
+        </is>
+      </c>
+      <c r="D423" s="249" t="inlineStr">
+        <is>
+          <t>Frutas de Temporada Jose</t>
+        </is>
+      </c>
+      <c r="E423" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Fruit</t>
+        </is>
+      </c>
+      <c r="F423" s="67" t="n">
+        <v>30</v>
+      </c>
+      <c r="G423" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H423" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I423" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J423" s="383" t="inlineStr">
+        <is>
+          <t>Solo melon $30; sin total impreso</t>
+        </is>
+      </c>
     </row>
     <row r="424">
-      <c r="B424" s="64" t="n"/>
-      <c r="C424" s="69" t="n"/>
-      <c r="D424" s="68" t="n"/>
-      <c r="E424" s="69" t="n"/>
-      <c r="F424" s="70" t="n"/>
-      <c r="G424" s="23" t="n"/>
-      <c r="H424" s="23" t="n"/>
-      <c r="I424" s="55" t="n"/>
+      <c r="B424" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C424" s="252" t="inlineStr">
+        <is>
+          <t>Morron surtido</t>
+        </is>
+      </c>
+      <c r="D424" s="253" t="inlineStr">
+        <is>
+          <t>Verduras Selectas Oscar</t>
+        </is>
+      </c>
+      <c r="E424" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F424" s="70" t="n">
+        <v>20</v>
+      </c>
+      <c r="G424" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H424" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I424" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J424" s="383" t="inlineStr">
+        <is>
+          <t>Morron $20; sin total impreso</t>
+        </is>
+      </c>
     </row>
     <row r="425">
-      <c r="B425" s="64" t="n"/>
-      <c r="C425" s="65" t="n"/>
-      <c r="D425" s="66" t="n"/>
-      <c r="E425" s="65" t="n"/>
-      <c r="F425" s="67" t="n"/>
-      <c r="G425" s="14" t="n"/>
-      <c r="H425" s="14" t="n"/>
-      <c r="I425" s="43" t="n"/>
+      <c r="B425" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C425" s="248" t="inlineStr">
+        <is>
+          <t>Fresa 0.775kg @ $65/kg</t>
+        </is>
+      </c>
+      <c r="D425" s="249" t="inlineStr">
+        <is>
+          <t>Nota manuscrita</t>
+        </is>
+      </c>
+      <c r="E425" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Fruit</t>
+        </is>
+      </c>
+      <c r="F425" s="67" t="n">
+        <v>50</v>
+      </c>
+      <c r="G425" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H425" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I425" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J425" s="383" t="inlineStr">
+        <is>
+          <t>.775x65=50; efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="426">
-      <c r="B426" s="64" t="n"/>
-      <c r="C426" s="69" t="n"/>
-      <c r="D426" s="68" t="n"/>
-      <c r="E426" s="69" t="n"/>
-      <c r="F426" s="70" t="n"/>
-      <c r="G426" s="23" t="n"/>
-      <c r="H426" s="23" t="n"/>
-      <c r="I426" s="55" t="n"/>
+      <c r="B426" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C426" s="252" t="inlineStr">
+        <is>
+          <t>Gelatinas, hot cakes, jarabe, verduras congeladas</t>
+        </is>
+      </c>
+      <c r="D426" s="253" t="inlineStr">
+        <is>
+          <t>Basicos</t>
+        </is>
+      </c>
+      <c r="E426" s="252" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F426" s="70" t="n">
+        <v>354.5</v>
+      </c>
+      <c r="G426" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H426" s="254" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I426" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J426" s="383" t="inlineStr">
+        <is>
+          <t>Total $358 - desc $3.50 = $354.50; tarjeta</t>
+        </is>
+      </c>
     </row>
     <row r="427">
-      <c r="B427" s="64" t="n"/>
-      <c r="C427" s="65" t="n"/>
-      <c r="D427" s="66" t="n"/>
-      <c r="E427" s="65" t="n"/>
-      <c r="F427" s="67" t="n"/>
-      <c r="G427" s="14" t="n"/>
-      <c r="H427" s="14" t="n"/>
-      <c r="I427" s="43" t="n"/>
+      <c r="B427" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C427" s="248" t="inlineStr">
+        <is>
+          <t>Melocoton 2.5kg + Platano</t>
+        </is>
+      </c>
+      <c r="D427" s="249" t="inlineStr">
+        <is>
+          <t>Remision</t>
+        </is>
+      </c>
+      <c r="E427" s="248" t="inlineStr">
+        <is>
+          <t>Ingredients - Fruit</t>
+        </is>
+      </c>
+      <c r="F427" s="67" t="n">
+        <v>68</v>
+      </c>
+      <c r="G427" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H427" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I427" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J427" s="383" t="inlineStr">
+        <is>
+          <t>Melocoton $50 + platano $18 = $68; efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="428">
-      <c r="B428" s="64" t="n"/>
-      <c r="C428" s="69" t="n"/>
-      <c r="D428" s="68" t="n"/>
-      <c r="E428" s="69" t="n"/>
-      <c r="F428" s="70" t="n"/>
-      <c r="G428" s="23" t="n"/>
-      <c r="H428" s="23" t="n"/>
-      <c r="I428" s="55" t="n"/>
+      <c r="B428" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C428" s="252" t="inlineStr">
+        <is>
+          <t>Papaya</t>
+        </is>
+      </c>
+      <c r="D428" s="253" t="inlineStr">
+        <is>
+          <t>Remision</t>
+        </is>
+      </c>
+      <c r="E428" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Fruit</t>
+        </is>
+      </c>
+      <c r="F428" s="70" t="n">
+        <v>36</v>
+      </c>
+      <c r="G428" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H428" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I428" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J428" s="383" t="inlineStr">
+        <is>
+          <t>Papaya total $36; efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="429">
-      <c r="B429" s="64" t="n"/>
-      <c r="C429" s="65" t="n"/>
-      <c r="D429" s="66" t="n"/>
-      <c r="E429" s="65" t="n"/>
-      <c r="F429" s="67" t="n"/>
-      <c r="G429" s="14" t="n"/>
-      <c r="H429" s="14" t="n"/>
-      <c r="I429" s="43" t="n"/>
+      <c r="B429" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C429" s="248" t="inlineStr">
+        <is>
+          <t>Granola 400g + Tortillas blancas 4.435kg</t>
+        </is>
+      </c>
+      <c r="D429" s="249" t="inlineStr">
+        <is>
+          <t>Chedraui Selecto</t>
+        </is>
+      </c>
+      <c r="E429" s="248" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F429" s="67" t="n">
+        <v>108.43</v>
+      </c>
+      <c r="G429" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H429" s="250" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="I429" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J429" s="383" t="inlineStr">
+        <is>
+          <t>Granola $53 + tortillas $55.43; debito ***0311</t>
+        </is>
+      </c>
     </row>
     <row r="430">
-      <c r="B430" s="64" t="n"/>
-      <c r="C430" s="69" t="n"/>
-      <c r="D430" s="68" t="n"/>
-      <c r="E430" s="69" t="n"/>
-      <c r="F430" s="70" t="n"/>
-      <c r="G430" s="23" t="n"/>
-      <c r="H430" s="23" t="n"/>
-      <c r="I430" s="55" t="n"/>
+      <c r="B430" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C430" s="252" t="inlineStr">
+        <is>
+          <t>Jitomate 8.3kg + Aguacate Hass</t>
+        </is>
+      </c>
+      <c r="D430" s="253" t="inlineStr">
+        <is>
+          <t>Frutas Finas Ana Pao</t>
+        </is>
+      </c>
+      <c r="E430" s="252" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F430" s="70" t="n">
+        <v>126</v>
+      </c>
+      <c r="G430" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H430" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I430" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J430" s="383" t="inlineStr">
+        <is>
+          <t>Jitomate $100 + hass $26 = $126; sin total impreso</t>
+        </is>
+      </c>
     </row>
     <row r="431">
-      <c r="B431" s="64" t="n"/>
-      <c r="C431" s="65" t="n"/>
-      <c r="D431" s="66" t="n"/>
-      <c r="E431" s="65" t="n"/>
-      <c r="F431" s="67" t="n"/>
-      <c r="G431" s="14" t="n"/>
-      <c r="H431" s="14" t="n"/>
-      <c r="I431" s="43" t="n"/>
+      <c r="B431" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C431" s="248" t="inlineStr">
+        <is>
+          <t>John — Head Chef Week 7</t>
+        </is>
+      </c>
+      <c r="D431" s="249" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E431" s="248" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F431" s="67" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G431" s="250" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H431" s="250" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I431" s="251" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J431" s="383" t="inlineStr">
+        <is>
+          <t>Week 7 salary, paid Saturday 04 Jul (usual $3,750; $50 higher this week)</t>
+        </is>
+      </c>
     </row>
     <row r="432">
-      <c r="B432" s="64" t="n"/>
-      <c r="C432" s="69" t="n"/>
-      <c r="D432" s="68" t="n"/>
-      <c r="E432" s="69" t="n"/>
-      <c r="F432" s="70" t="n"/>
-      <c r="G432" s="23" t="n"/>
-      <c r="H432" s="23" t="n"/>
-      <c r="I432" s="55" t="n"/>
+      <c r="B432" s="382" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C432" s="252" t="inlineStr">
+        <is>
+          <t>Duvi/Debi — Limpieza Week 7 (5 days)</t>
+        </is>
+      </c>
+      <c r="D432" s="253" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E432" s="252" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F432" s="70" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G432" s="254" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H432" s="254" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I432" s="255" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J432" s="383" t="inlineStr">
+        <is>
+          <t>Week 7, worked 5 days @ $250/day = $1,250, paid Saturday 04 Jul</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="B433" s="64" t="n"/>
@@ -44435,7 +44999,7 @@
     <row r="20">
       <c r="A20" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Pantry</t>
+          <t>Ingredients - Vegetables</t>
         </is>
       </c>
       <c r="B20" s="378">
@@ -44462,7 +45026,7 @@
     <row r="21">
       <c r="A21" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Vegetables</t>
+          <t>Ingredients - Pantry</t>
         </is>
       </c>
       <c r="B21" s="378">
@@ -44759,7 +45323,7 @@
     <row r="32">
       <c r="A32" s="380" t="inlineStr">
         <is>
-          <t>Software / Subscription</t>
+          <t>Supermarket/General</t>
         </is>
       </c>
       <c r="B32" s="378">
@@ -44786,7 +45350,7 @@
     <row r="33">
       <c r="A33" s="380" t="inlineStr">
         <is>
-          <t>Supermarket/General</t>
+          <t>Software / Subscription</t>
         </is>
       </c>
       <c r="B33" s="378">
@@ -44975,7 +45539,7 @@
     <row r="40">
       <c r="A40" s="380" t="inlineStr">
         <is>
-          <t>Staff - Propinas</t>
+          <t>Packaging/Disposables</t>
         </is>
       </c>
       <c r="B40" s="378">
@@ -45002,7 +45566,7 @@
     <row r="41">
       <c r="A41" s="380" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Staff - Propinas</t>
         </is>
       </c>
       <c r="B41" s="378">
@@ -45029,7 +45593,7 @@
     <row r="42">
       <c r="A42" s="380" t="inlineStr">
         <is>
-          <t>Ingredients - Produce</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="B42" s="378">
@@ -45054,21 +45618,21 @@
       <c r="L42" s="374" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="377" t="inlineStr">
-        <is>
-          <t>TOTAL EXPENSES</t>
-        </is>
-      </c>
-      <c r="B43" s="379">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
-        <v/>
-      </c>
-      <c r="C43" s="379">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
-        <v/>
-      </c>
-      <c r="D43" s="379">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+      <c r="A43" s="380" t="inlineStr">
+        <is>
+          <t>Ingredients - Produce</t>
+        </is>
+      </c>
+      <c r="B43" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A43,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C43" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A43,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <v/>
+      </c>
+      <c r="D43" s="378">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A43,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E43" s="374" t="n"/>
@@ -45083,19 +45647,19 @@
     <row r="44">
       <c r="A44" s="377" t="inlineStr">
         <is>
-          <t>NET PROFIT / LOSS</t>
+          <t>TOTAL EXPENSES</t>
         </is>
       </c>
       <c r="B44" s="379">
-        <f>B4-B43</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C44" s="379">
-        <f>C4-C43</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D44" s="379">
-        <f>D4-D43</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E44" s="374" t="n"/>
@@ -45108,10 +45672,23 @@
       <c r="L44" s="374" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="374" t="n"/>
-      <c r="B45" s="374" t="n"/>
-      <c r="C45" s="374" t="n"/>
-      <c r="D45" s="374" t="n"/>
+      <c r="A45" s="377" t="inlineStr">
+        <is>
+          <t>NET PROFIT / LOSS</t>
+        </is>
+      </c>
+      <c r="B45" s="379">
+        <f>B4-B44</f>
+        <v/>
+      </c>
+      <c r="C45" s="379">
+        <f>C4-C44</f>
+        <v/>
+      </c>
+      <c r="D45" s="379">
+        <f>D4-D44</f>
+        <v/>
+      </c>
       <c r="E45" s="374" t="n"/>
       <c r="F45" s="374" t="n"/>
       <c r="G45" s="374" t="n"/>

</xml_diff>

<commit_message>
fixed an issue with Dashboard
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -21085,8 +21085,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -50636,14 +50636,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="313">
-      <c r="A1" s="417" t="inlineStr">
+      <c r="A1" s="407" t="inlineStr">
         <is>
           <t>LOKA — MONTHLY P&amp;L   (live formulas — auto-updates from Daily Log &amp; Expenses)</t>
         </is>
       </c>
-      <c r="B1" s="418" t="n"/>
-      <c r="C1" s="418" t="n"/>
-      <c r="D1" s="418" t="n"/>
+      <c r="B1" s="408" t="n"/>
+      <c r="C1" s="408" t="n"/>
+      <c r="D1" s="408" t="n"/>
       <c r="E1" s="409" t="n"/>
       <c r="F1" s="409" t="n"/>
       <c r="G1" s="409" t="n"/>

</xml_diff>

<commit_message>
corrected few more issues
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5395,7 +5395,7 @@
         </is>
       </c>
       <c r="C143" s="283">
-        <f>SUM('📅 Daily Log'!D8:D500)+SUM('📅 Daily Log'!E8:E500)+SUM('📅 Daily Log'!G8:G500)</f>
+        <f>SUM('📅 Daily Log'!D8:D5000)+SUM('📅 Daily Log'!E8:E5000)+SUM('📅 Daily Log'!G8:G5000)</f>
         <v/>
       </c>
       <c r="D143" s="191" t="n"/>
@@ -5410,7 +5410,7 @@
         </is>
       </c>
       <c r="C144" s="283">
-        <f>SUM('💸 Expenses'!F8:F500)</f>
+        <f>SUM('💸 Expenses'!F8:F50000)</f>
         <v/>
       </c>
       <c r="D144" s="191" t="n"/>
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="C145" s="268">
-        <f>SUM('📅 Daily Log'!R8:R500)</f>
+        <f>SUM('📅 Daily Log'!R8:R5000)</f>
         <v/>
       </c>
     </row>
@@ -7587,7 +7587,7 @@
       </c>
       <c r="C17" s="333" t="n"/>
       <c r="D17" s="363">
-        <f>IFERROR(SUMPRODUCT((ISNUMBER('📅 Daily Log'!$B$8:$B$500))*('📅 Daily Log'!$B$8:$B$500&gt;=TODAY()-MOD(TODAY()-2,7))*('📅 Daily Log'!$B$8:$B$500&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER('📅 Daily Log'!$G$8:$G$500),'📅 Daily Log'!$G$8:$G$500,0)),0)</f>
+        <f>IFERROR(SUMPRODUCT((ISNUMBER('📅 Daily Log'!$B$8:$B$5000))*('📅 Daily Log'!$B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*('📅 Daily Log'!$B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER('📅 Daily Log'!$G$8:$G$5000),'📅 Daily Log'!$G$8:$G$5000,0)),0)</f>
         <v/>
       </c>
       <c r="E17" s="333" t="n"/>
@@ -9172,15 +9172,15 @@
       <c r="D6" s="28" t="n"/>
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
-        <f>SUMIFS($D$8:$D$500,$B$8:$B$500,TODAY())+SUMIFS($E$8:$E$500,$B$8:$B$500,TODAY())+SUMIFS($G$8:$G$500,$B$8:$B$500,TODAY())</f>
+        <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
         <v/>
       </c>
       <c r="G6" s="31">
-        <f>SUMIFS($G$8:$G$500,$B$8:$B$500,TODAY())</f>
+        <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
         <v/>
       </c>
       <c r="H6" s="28">
-        <f>SUMIFS($H$8:$H$500,$B$8:$B$500,TODAY())</f>
+        <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
         <v/>
       </c>
       <c r="I6" s="32">
@@ -9194,19 +9194,19 @@
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
-        <f>SUMPRODUCT((ISNUMBER($B$8:$B$500))*($B$8:$B$500&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$500&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$500),$F$8:$F$500,0))</f>
+        <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
         <v/>
       </c>
       <c r="N6" s="33">
-        <f>SUMPRODUCT((ISNUMBER($B$8:$B$500))*($B$8:$B$500&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$500&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$500),$F$8:$F$500,0))</f>
+        <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
         <v/>
       </c>
       <c r="O6" s="33">
-        <f>SUMPRODUCT((ISNUMBER($B$8:$B$500))*(MONTH($B$8:$B$500)=MONTH(TODAY()))*(YEAR($B$8:$B$500)=YEAR(TODAY()))*IF(ISNUMBER($F$8:$F$500),$F$8:$F$500,0))</f>
+        <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*(MONTH($B$8:$B$5000)=MONTH(TODAY()))*(YEAR($B$8:$B$5000)=YEAR(TODAY()))*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
         <v/>
       </c>
       <c r="P6">
-        <f>SUMPRODUCT((ISNUMBER($B$8:$B$500))*($B$8:$B$500&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$500&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($H$8:$H$500),$H$8:$H$500,0))</f>
+        <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($H$8:$H$5000),$H$8:$H$5000,0))</f>
         <v/>
       </c>
       <c r="Q6">
@@ -9362,20 +9362,20 @@
       </c>
       <c r="F8" s="38">
         <f>IFERROR(D8+E8+G8,0)</f>
-        <v>3689.0</v>
+        <v/>
       </c>
       <c r="G8" s="39" t="n"/>
       <c r="H8" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B8,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B8+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B8,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B8+1))</f>
         <v/>
       </c>
       <c r="I8" s="41">
         <f>IFERROR(F8-H8,0)</f>
-        <v>1060.0</v>
+        <v/>
       </c>
       <c r="J8" s="42">
         <f>IFERROR(I8/F8,0)</f>
-        <v>0.287341</v>
+        <v/>
       </c>
       <c r="K8" s="43" t="n"/>
       <c r="L8" s="9" t="inlineStr">
@@ -9420,20 +9420,20 @@
       </c>
       <c r="F9" s="50">
         <f>IFERROR(D9+E9+G9,0)</f>
-        <v>3854.0</v>
+        <v/>
       </c>
       <c r="G9" s="51" t="n"/>
       <c r="H9" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B9,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B9+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B9,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B9+1))</f>
         <v/>
       </c>
       <c r="I9" s="53">
         <f>IFERROR(F9-H9,0)</f>
-        <v>3824.0</v>
+        <v/>
       </c>
       <c r="J9" s="54">
         <f>IFERROR(I9/F9,0)</f>
-        <v>0.992216</v>
+        <v/>
       </c>
       <c r="K9" s="55" t="n"/>
       <c r="L9" s="18" t="inlineStr">
@@ -9478,20 +9478,20 @@
       </c>
       <c r="F10" s="38">
         <f>IFERROR(D10+E10+G10,0)</f>
-        <v>4124.0</v>
+        <v/>
       </c>
       <c r="G10" s="39" t="n"/>
       <c r="H10" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B10,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B10+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B10,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B10+1))</f>
         <v/>
       </c>
       <c r="I10" s="41">
         <f>IFERROR(F10-H10,0)</f>
-        <v>347.0</v>
+        <v/>
       </c>
       <c r="J10" s="42">
         <f>IFERROR(I10/F10,0)</f>
-        <v>0.084142</v>
+        <v/>
       </c>
       <c r="K10" s="43" t="n"/>
       <c r="L10" s="9" t="inlineStr">
@@ -9536,20 +9536,20 @@
       </c>
       <c r="F11" s="50">
         <f>IFERROR(D11+E11+G11,0)</f>
-        <v>4733.0</v>
+        <v/>
       </c>
       <c r="G11" s="51" t="n"/>
       <c r="H11" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B11,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B11+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B11,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B11+1))</f>
         <v/>
       </c>
       <c r="I11" s="53">
         <f>IFERROR(F11-H11,0)</f>
-        <v>2299.0</v>
+        <v/>
       </c>
       <c r="J11" s="54">
         <f>IFERROR(I11/F11,0)</f>
-        <v>0.485738</v>
+        <v/>
       </c>
       <c r="K11" s="55" t="n"/>
       <c r="L11" s="18" t="inlineStr">
@@ -9594,20 +9594,20 @@
       </c>
       <c r="F12" s="38">
         <f>IFERROR(D12+E12+G12,0)</f>
-        <v>4282.0</v>
+        <v/>
       </c>
       <c r="G12" s="39" t="n"/>
       <c r="H12" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B12,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B12+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B12,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B12+1))</f>
         <v/>
       </c>
       <c r="I12" s="41">
         <f>IFERROR(F12-H12,0)</f>
-        <v>2825.0</v>
+        <v/>
       </c>
       <c r="J12" s="42">
         <f>IFERROR(I12/F12,0)</f>
-        <v>0.659738</v>
+        <v/>
       </c>
       <c r="K12" s="43" t="n"/>
       <c r="L12" s="9" t="inlineStr">
@@ -9652,20 +9652,20 @@
       </c>
       <c r="F13" s="50">
         <f>IFERROR(D13+E13+G13,0)</f>
-        <v>3802.0</v>
+        <v/>
       </c>
       <c r="G13" s="51" t="n"/>
       <c r="H13" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B13,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B13+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B13,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B13+1))</f>
         <v/>
       </c>
       <c r="I13" s="53">
         <f>IFERROR(F13-H13,0)</f>
-        <v>-3953.43</v>
+        <v/>
       </c>
       <c r="J13" s="54">
         <f>IFERROR(I13/F13,0)</f>
-        <v>-1.039829</v>
+        <v/>
       </c>
       <c r="K13" s="55" t="inlineStr">
         <is>
@@ -9712,20 +9712,20 @@
       </c>
       <c r="F14" s="38">
         <f>IFERROR(D14+E14+G14,0)</f>
-        <v>1198.0</v>
+        <v/>
       </c>
       <c r="G14" s="39" t="n"/>
       <c r="H14" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B14,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B14+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B14,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B14+1))</f>
         <v/>
       </c>
       <c r="I14" s="41">
         <f>IFERROR(F14-H14,0)</f>
-        <v>122.0</v>
+        <v/>
       </c>
       <c r="J14" s="42">
         <f>IFERROR(I14/F14,0)</f>
-        <v>0.101836</v>
+        <v/>
       </c>
       <c r="K14" s="43" t="inlineStr">
         <is>
@@ -9774,20 +9774,20 @@
       </c>
       <c r="F15" s="50">
         <f>IFERROR(D15+E15+G15,0)</f>
-        <v>3730.0</v>
+        <v/>
       </c>
       <c r="G15" s="51" t="n"/>
       <c r="H15" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B15,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B15+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B15,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B15+1))</f>
         <v/>
       </c>
       <c r="I15" s="53">
         <f>IFERROR(F15-H15,0)</f>
-        <v>708.55</v>
+        <v/>
       </c>
       <c r="J15" s="54">
         <f>IFERROR(I15/F15,0)</f>
-        <v>0.18996</v>
+        <v/>
       </c>
       <c r="K15" s="55" t="n"/>
       <c r="L15" s="18" t="inlineStr">
@@ -9832,20 +9832,20 @@
       </c>
       <c r="F16" s="38">
         <f>IFERROR(D16+E16+G16,0)</f>
-        <v>4264.0</v>
+        <v/>
       </c>
       <c r="G16" s="39" t="n"/>
       <c r="H16" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B16,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B16+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B16,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B16+1))</f>
         <v/>
       </c>
       <c r="I16" s="41">
         <f>IFERROR(F16-H16,0)</f>
-        <v>3072.4</v>
+        <v/>
       </c>
       <c r="J16" s="42">
         <f>IFERROR(I16/F16,0)</f>
-        <v>0.720544</v>
+        <v/>
       </c>
       <c r="K16" s="43" t="n"/>
       <c r="L16" s="9" t="inlineStr">
@@ -9890,20 +9890,20 @@
       </c>
       <c r="F17" s="50">
         <f>IFERROR(D17+E17+G17,0)</f>
-        <v>3621.0</v>
+        <v/>
       </c>
       <c r="G17" s="51" t="n"/>
       <c r="H17" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B17,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B17+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B17,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B17+1))</f>
         <v/>
       </c>
       <c r="I17" s="53">
         <f>IFERROR(F17-H17,0)</f>
-        <v>2547.78</v>
+        <v/>
       </c>
       <c r="J17" s="54">
         <f>IFERROR(I17/F17,0)</f>
-        <v>0.703612</v>
+        <v/>
       </c>
       <c r="K17" s="55" t="n"/>
       <c r="L17" s="18" t="inlineStr">
@@ -9948,20 +9948,20 @@
       </c>
       <c r="F18" s="38">
         <f>IFERROR(D18+E18+G18,0)</f>
-        <v>4070.0</v>
+        <v/>
       </c>
       <c r="G18" s="39" t="n"/>
       <c r="H18" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B18,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B18+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B18,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B18+1))</f>
         <v/>
       </c>
       <c r="I18" s="41">
         <f>IFERROR(F18-H18,0)</f>
-        <v>2138.66</v>
+        <v/>
       </c>
       <c r="J18" s="42">
         <f>IFERROR(I18/F18,0)</f>
-        <v>0.525469</v>
+        <v/>
       </c>
       <c r="K18" s="43" t="n"/>
       <c r="L18" s="9" t="inlineStr">
@@ -10006,20 +10006,20 @@
       </c>
       <c r="F19" s="50">
         <f>IFERROR(D19+E19+G19,0)</f>
-        <v>6086.0</v>
+        <v/>
       </c>
       <c r="G19" s="51" t="n"/>
       <c r="H19" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B19,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B19+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B19,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B19+1))</f>
         <v/>
       </c>
       <c r="I19" s="53">
         <f>IFERROR(F19-H19,0)</f>
-        <v>5828.71</v>
+        <v/>
       </c>
       <c r="J19" s="54">
         <f>IFERROR(I19/F19,0)</f>
-        <v>0.957724</v>
+        <v/>
       </c>
       <c r="K19" s="55" t="n"/>
       <c r="L19" s="18" t="inlineStr">
@@ -10064,20 +10064,20 @@
       </c>
       <c r="F20" s="38">
         <f>IFERROR(D20+E20+G20,0)</f>
-        <v>4603.0</v>
+        <v/>
       </c>
       <c r="G20" s="39" t="n"/>
       <c r="H20" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B20,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B20+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B20,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B20+1))</f>
         <v/>
       </c>
       <c r="I20" s="41">
         <f>IFERROR(F20-H20,0)</f>
-        <v>-1371.3</v>
+        <v/>
       </c>
       <c r="J20" s="42">
         <f>IFERROR(I20/F20,0)</f>
-        <v>-0.297914</v>
+        <v/>
       </c>
       <c r="K20" s="43" t="n"/>
       <c r="L20" s="9" t="inlineStr">
@@ -10120,20 +10120,20 @@
       </c>
       <c r="F21" s="50">
         <f>IFERROR(D21+E21+G21,0)</f>
-        <v>893.0</v>
+        <v/>
       </c>
       <c r="G21" s="51" t="n"/>
       <c r="H21" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B21,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B21+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B21,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B21+1))</f>
         <v/>
       </c>
       <c r="I21" s="53">
         <f>IFERROR(F21-H21,0)</f>
-        <v>-9419.0</v>
+        <v/>
       </c>
       <c r="J21" s="54">
         <f>IFERROR(I21/F21,0)</f>
-        <v>-10.547592</v>
+        <v/>
       </c>
       <c r="K21" s="55" t="n"/>
       <c r="L21" s="18" t="inlineStr">
@@ -10178,22 +10178,22 @@
       </c>
       <c r="F22" s="38">
         <f>IFERROR(D22+E22+G22,0)</f>
-        <v>5019.0</v>
+        <v/>
       </c>
       <c r="G22" s="39" t="n">
         <v>310</v>
       </c>
       <c r="H22" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B22,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B22+1))</f>
-        <v>5329.64</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B22,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B22+1))</f>
+        <v/>
       </c>
       <c r="I22" s="41">
         <f>IFERROR(F22-H22,0)</f>
-        <v>-310.64</v>
+        <v/>
       </c>
       <c r="J22" s="42">
         <f>IFERROR(I22/F22,0)</f>
-        <v>-0.061893</v>
+        <v/>
       </c>
       <c r="K22" s="43" t="n"/>
       <c r="L22" s="9" t="inlineStr">
@@ -10238,22 +10238,22 @@
       </c>
       <c r="F23" s="50">
         <f>IFERROR(D23+E23+G23,0)</f>
-        <v>1843.0</v>
+        <v/>
       </c>
       <c r="G23" s="51" t="n">
         <v>283</v>
       </c>
       <c r="H23" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B23,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B23+1))</f>
-        <v>2379.11</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B23,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B23+1))</f>
+        <v/>
       </c>
       <c r="I23" s="53">
         <f>IFERROR(F23-H23,0)</f>
-        <v>-536.11</v>
+        <v/>
       </c>
       <c r="J23" s="54">
         <f>IFERROR(I23/F23,0)</f>
-        <v>-0.29089</v>
+        <v/>
       </c>
       <c r="K23" s="55" t="n"/>
       <c r="L23" s="18" t="inlineStr">
@@ -10298,22 +10298,22 @@
       </c>
       <c r="F24" s="38">
         <f>IFERROR(D24+E24+G24,0)</f>
-        <v>3912.0</v>
+        <v/>
       </c>
       <c r="G24" s="39" t="n">
         <v>120</v>
       </c>
       <c r="H24" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B24,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B24+1))</f>
-        <v>4211.86</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B24,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B24+1))</f>
+        <v/>
       </c>
       <c r="I24" s="41">
         <f>IFERROR(F24-H24,0)</f>
-        <v>-299.86</v>
+        <v/>
       </c>
       <c r="J24" s="42">
         <f>IFERROR(I24/F24,0)</f>
-        <v>-0.076651</v>
+        <v/>
       </c>
       <c r="K24" s="43" t="n"/>
       <c r="L24" s="9" t="inlineStr">
@@ -10358,20 +10358,20 @@
       </c>
       <c r="F25" s="50">
         <f>IFERROR(D25+E25+G25,0)</f>
-        <v>3757.0</v>
+        <v/>
       </c>
       <c r="G25" s="51" t="n"/>
       <c r="H25" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B25,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B25+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B25,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B25+1))</f>
         <v/>
       </c>
       <c r="I25" s="53">
         <f>IFERROR(F25-H25,0)</f>
-        <v>-17202.96</v>
+        <v/>
       </c>
       <c r="J25" s="54">
         <f>IFERROR(I25/F25,0)</f>
-        <v>-4.578909</v>
+        <v/>
       </c>
       <c r="K25" s="55" t="n"/>
       <c r="L25" s="18" t="inlineStr">
@@ -10416,22 +10416,22 @@
       </c>
       <c r="F26" s="38">
         <f>IFERROR(D26+E26+G26,0)</f>
-        <v>4408.0</v>
+        <v/>
       </c>
       <c r="G26" s="39" t="n">
         <v>135</v>
       </c>
       <c r="H26" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B26,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B26+1))</f>
-        <v>878.06</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B26,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B26+1))</f>
+        <v/>
       </c>
       <c r="I26" s="41">
         <f>IFERROR(F26-H26,0)</f>
-        <v>3529.94</v>
+        <v/>
       </c>
       <c r="J26" s="42">
         <f>IFERROR(I26/F26,0)</f>
-        <v>0.800803</v>
+        <v/>
       </c>
       <c r="K26" s="43" t="n"/>
       <c r="L26" s="9" t="inlineStr">
@@ -10476,20 +10476,20 @@
       </c>
       <c r="F27" s="50">
         <f>IFERROR(D27+E27+G27,0)</f>
-        <v>2334.0</v>
+        <v/>
       </c>
       <c r="G27" s="51" t="n"/>
       <c r="H27" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B27,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B27+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B27,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B27+1))</f>
         <v/>
       </c>
       <c r="I27" s="53">
         <f>IFERROR(F27-H27,0)</f>
-        <v>-3080.0</v>
+        <v/>
       </c>
       <c r="J27" s="54">
         <f>IFERROR(I27/F27,0)</f>
-        <v>-1.319623</v>
+        <v/>
       </c>
       <c r="K27" s="55" t="n"/>
       <c r="L27" s="18" t="inlineStr">
@@ -10534,12 +10534,12 @@
       </c>
       <c r="G28" s="39" t="n"/>
       <c r="H28" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B28,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B28+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B28,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B28+1))</f>
         <v/>
       </c>
       <c r="I28" s="41">
         <f>IFERROR(F28-H28,0)</f>
-        <v>-1671.0</v>
+        <v/>
       </c>
       <c r="J28" s="42" t="n"/>
       <c r="K28" s="43" t="n"/>
@@ -10585,22 +10585,22 @@
       </c>
       <c r="F29" s="50">
         <f>IFERROR(D29+E29+G29,0)</f>
-        <v>3727.0</v>
+        <v/>
       </c>
       <c r="G29" s="51" t="n">
         <v>99</v>
       </c>
       <c r="H29" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B29,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B29+1))</f>
-        <v>3187.11</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B29,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B29+1))</f>
+        <v/>
       </c>
       <c r="I29" s="53">
         <f>IFERROR(F29-H29,0)</f>
-        <v>539.89</v>
+        <v/>
       </c>
       <c r="J29" s="54">
         <f>IFERROR(I29/F29,0)</f>
-        <v>0.144859</v>
+        <v/>
       </c>
       <c r="K29" s="55" t="n"/>
       <c r="L29" s="18" t="inlineStr">
@@ -10645,20 +10645,20 @@
       </c>
       <c r="F30" s="38">
         <f>IFERROR(D30+E30+G30,0)</f>
-        <v>5410.0</v>
+        <v/>
       </c>
       <c r="G30" s="39" t="n"/>
       <c r="H30" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B30,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B30+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B30,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B30+1))</f>
         <v/>
       </c>
       <c r="I30" s="41">
         <f>IFERROR(F30-H30,0)</f>
-        <v>-1213.98</v>
+        <v/>
       </c>
       <c r="J30" s="42">
         <f>IFERROR(I30/F30,0)</f>
-        <v>-0.224396</v>
+        <v/>
       </c>
       <c r="K30" s="43" t="n"/>
       <c r="L30" s="9" t="inlineStr">
@@ -10703,20 +10703,20 @@
       </c>
       <c r="F31" s="50">
         <f>IFERROR(D31+E31+G31,0)</f>
-        <v>4265.0</v>
+        <v/>
       </c>
       <c r="G31" s="51" t="n"/>
       <c r="H31" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B31,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B31+1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B31,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B31+1))</f>
         <v/>
       </c>
       <c r="I31" s="53">
         <f>IFERROR(F31-H31,0)</f>
-        <v>2923.19</v>
+        <v/>
       </c>
       <c r="J31" s="54">
         <f>IFERROR(I31/F31,0)</f>
-        <v>0.68539</v>
+        <v/>
       </c>
       <c r="K31" s="55" t="n"/>
       <c r="L31" s="18" t="inlineStr">
@@ -10761,22 +10761,22 @@
       </c>
       <c r="F32" s="38">
         <f>IFERROR(D32+E32+G32,0)</f>
-        <v>4166.0</v>
+        <v/>
       </c>
       <c r="G32" s="39" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B32,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B32+1))</f>
-        <v>4044.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B32,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B32+1))</f>
+        <v/>
       </c>
       <c r="I32" s="41">
         <f>IFERROR(F32-H32,0)</f>
-        <v>122.0</v>
+        <v/>
       </c>
       <c r="J32" s="42">
         <f>IFERROR(I32/F32,0)</f>
-        <v>0.029285</v>
+        <v/>
       </c>
       <c r="K32" s="43" t="n"/>
       <c r="L32" s="9" t="inlineStr">
@@ -10821,22 +10821,22 @@
       </c>
       <c r="F33" s="50">
         <f>IFERROR(D33+E33+G33,0)</f>
-        <v>6070.0</v>
+        <v/>
       </c>
       <c r="G33" s="51" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B33,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B33+1))</f>
-        <v>901.8</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B33,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B33+1))</f>
+        <v/>
       </c>
       <c r="I33" s="53">
         <f>IFERROR(F33-H33,0)</f>
-        <v>5168.2</v>
+        <v/>
       </c>
       <c r="J33" s="54">
         <f>IFERROR(I33/F33,0)</f>
-        <v>0.851433</v>
+        <v/>
       </c>
       <c r="K33" s="55" t="n"/>
       <c r="L33" s="18" t="inlineStr">
@@ -10881,22 +10881,22 @@
       </c>
       <c r="F34" s="38">
         <f>IFERROR(D34+E34+G34,0)</f>
-        <v>1811.0</v>
+        <v/>
       </c>
       <c r="G34" s="39" t="n">
         <v>0</v>
       </c>
       <c r="H34" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B34,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B34+1))</f>
-        <v>8084.16</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B34,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B34+1))</f>
+        <v/>
       </c>
       <c r="I34" s="41">
         <f>IFERROR(F34-H34,0)</f>
-        <v>-6273.16</v>
+        <v/>
       </c>
       <c r="J34" s="42">
         <f>IFERROR(I34/F34,0)</f>
-        <v>-3.46392</v>
+        <v/>
       </c>
       <c r="K34" s="43" t="n"/>
       <c r="L34" s="9" t="inlineStr">
@@ -10941,22 +10941,22 @@
       </c>
       <c r="F35" s="50">
         <f>IFERROR(D35+E35+G35,0)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="G35" s="51" t="n">
         <v>0</v>
       </c>
       <c r="H35" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B35,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B35+1))</f>
-        <v>1526.18</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B35,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B35+1))</f>
+        <v/>
       </c>
       <c r="I35" s="53">
         <f>IFERROR(F35-H35,0)</f>
-        <v>-1526.18</v>
+        <v/>
       </c>
       <c r="J35" s="54">
         <f>IFERROR(I35/F35,0)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K35" s="55" t="n"/>
       <c r="L35" s="18" t="inlineStr">
@@ -11001,22 +11001,22 @@
       </c>
       <c r="F36" s="38">
         <f>IFERROR(D36+E36+G36,0)</f>
-        <v>4423.0</v>
+        <v/>
       </c>
       <c r="G36" s="39" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B36,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B36+1))</f>
-        <v>2858.08</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B36,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B36+1))</f>
+        <v/>
       </c>
       <c r="I36" s="41">
         <f>IFERROR(F36-H36,0)</f>
-        <v>1564.92</v>
+        <v/>
       </c>
       <c r="J36" s="42">
         <f>IFERROR(I36/F36,0)</f>
-        <v>0.353814</v>
+        <v/>
       </c>
       <c r="K36" s="43" t="n"/>
       <c r="L36" s="9" t="inlineStr">
@@ -11061,22 +11061,22 @@
       </c>
       <c r="F37" s="50">
         <f>IFERROR(D37+E37+G37,0)</f>
-        <v>2786.0</v>
+        <v/>
       </c>
       <c r="G37" s="51" t="n">
         <v>0</v>
       </c>
       <c r="H37" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B37,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B37+1))</f>
-        <v>2541.9</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B37,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B37+1))</f>
+        <v/>
       </c>
       <c r="I37" s="53">
         <f>IFERROR(F37-H37,0)</f>
-        <v>244.1</v>
+        <v/>
       </c>
       <c r="J37" s="54">
         <f>IFERROR(I37/F37,0)</f>
-        <v>0.087617</v>
+        <v/>
       </c>
       <c r="K37" s="55" t="n"/>
       <c r="L37" s="18" t="inlineStr">
@@ -11121,22 +11121,22 @@
       </c>
       <c r="F38" s="38">
         <f>IFERROR(D38+E38+G38,0)</f>
-        <v>4404.0</v>
+        <v/>
       </c>
       <c r="G38" s="39" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B38,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B38+1))</f>
-        <v>2353.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B38,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B38+1))</f>
+        <v/>
       </c>
       <c r="I38" s="41">
         <f>IFERROR(F38-H38,0)</f>
-        <v>2051.0</v>
+        <v/>
       </c>
       <c r="J38" s="42">
         <f>IFERROR(I38/F38,0)</f>
-        <v>0.465713</v>
+        <v/>
       </c>
       <c r="K38" s="43" t="n"/>
       <c r="L38" s="9" t="inlineStr">
@@ -11181,22 +11181,22 @@
       </c>
       <c r="F39" s="50">
         <f>IFERROR(D39+E39+G39,0)</f>
-        <v>4165.0</v>
+        <v/>
       </c>
       <c r="G39" s="51" t="n">
         <v>400</v>
       </c>
       <c r="H39" s="52">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B39,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B39+1))</f>
-        <v>2958.83</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B39,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B39+1))</f>
+        <v/>
       </c>
       <c r="I39" s="53">
         <f>IFERROR(F39-H39,0)</f>
-        <v>1206.17</v>
+        <v/>
       </c>
       <c r="J39" s="54">
         <f>IFERROR(I39/F39,0)</f>
-        <v>0.289597</v>
+        <v/>
       </c>
       <c r="K39" s="55" t="n"/>
       <c r="L39" s="18" t="inlineStr">
@@ -11241,22 +11241,22 @@
       </c>
       <c r="F40" s="38">
         <f>IFERROR(D40+E40+G40,0)</f>
-        <v>6804.0</v>
+        <v/>
       </c>
       <c r="G40" s="39" t="n">
         <v>120</v>
       </c>
       <c r="H40" s="40">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B40,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B40+1))</f>
-        <v>1483.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B40,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B40+1))</f>
+        <v/>
       </c>
       <c r="I40" s="41">
         <f>IFERROR(F40-H40,0)</f>
-        <v>5321.0</v>
+        <v/>
       </c>
       <c r="J40" s="42">
         <f>IFERROR(I40/F40,0)</f>
-        <v>0.78204</v>
+        <v/>
       </c>
       <c r="K40" s="43" t="n"/>
       <c r="L40" s="9" t="inlineStr">
@@ -11301,22 +11301,22 @@
       </c>
       <c r="F41" s="50">
         <f>IFERROR(D41+E41+G41,0)</f>
-        <v>2251.0</v>
+        <v/>
       </c>
       <c r="G41" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H41" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B41,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B41+1))</f>
-        <v>9320.81</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B41,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B41+1))</f>
+        <v/>
       </c>
       <c r="I41" s="259">
         <f>IFERROR(F41-H41,0)</f>
-        <v>-7069.81</v>
+        <v/>
       </c>
       <c r="J41" s="260">
         <f>IFERROR(I41/F41,0)</f>
-        <v>-3.140742</v>
+        <v/>
       </c>
       <c r="K41" s="254" t="n"/>
       <c r="L41" s="261" t="inlineStr">
@@ -11361,22 +11361,22 @@
       </c>
       <c r="F42" s="38">
         <f>IFERROR(D42+E42+G42,0)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="G42" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H42" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B42,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B42+1))</f>
-        <v>2065.85</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B42,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B42+1))</f>
+        <v/>
       </c>
       <c r="I42" s="274">
         <f>IFERROR(F42-H42,0)</f>
-        <v>-2065.85</v>
+        <v/>
       </c>
       <c r="J42" s="275">
         <f>IFERROR(I42/F42,0)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K42" s="250" t="n"/>
       <c r="L42" s="276" t="inlineStr">
@@ -11421,22 +11421,22 @@
       </c>
       <c r="F43" s="50">
         <f>IFERROR(D43+E43+G43,0)</f>
-        <v>4259.0</v>
+        <v/>
       </c>
       <c r="G43" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B43,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B43+1))</f>
-        <v>1451.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B43,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B43+1))</f>
+        <v/>
       </c>
       <c r="I43" s="259">
         <f>IFERROR(F43-H43,0)</f>
-        <v>2808.0</v>
+        <v/>
       </c>
       <c r="J43" s="260">
         <f>IFERROR(I43/F43,0)</f>
-        <v>0.65931</v>
+        <v/>
       </c>
       <c r="K43" s="254" t="n"/>
       <c r="L43" s="261" t="inlineStr">
@@ -11481,22 +11481,22 @@
       </c>
       <c r="F44" s="38">
         <f>IFERROR(D44+E44+G44,0)</f>
-        <v>2967.0</v>
+        <v/>
       </c>
       <c r="G44" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B44,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B44+1))</f>
-        <v>757.13</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B44,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B44+1))</f>
+        <v/>
       </c>
       <c r="I44" s="274">
         <f>IFERROR(F44-H44,0)</f>
-        <v>2209.87</v>
+        <v/>
       </c>
       <c r="J44" s="275">
         <f>IFERROR(I44/F44,0)</f>
-        <v>0.744816</v>
+        <v/>
       </c>
       <c r="K44" s="250" t="n"/>
       <c r="L44" s="276" t="inlineStr">
@@ -11541,22 +11541,22 @@
       </c>
       <c r="F45" s="50">
         <f>IFERROR(D45+E45+G45,0)</f>
-        <v>3589.0</v>
+        <v/>
       </c>
       <c r="G45" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H45" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B45,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B45+1))</f>
-        <v>3781.35</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B45,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B45+1))</f>
+        <v/>
       </c>
       <c r="I45" s="259">
         <f>IFERROR(F45-H45,0)</f>
-        <v>-192.35</v>
+        <v/>
       </c>
       <c r="J45" s="260">
         <f>IFERROR(I45/F45,0)</f>
-        <v>-0.053594</v>
+        <v/>
       </c>
       <c r="K45" s="254" t="n"/>
       <c r="L45" s="261" t="inlineStr">
@@ -11601,22 +11601,22 @@
       </c>
       <c r="F46" s="38">
         <f>IFERROR(D46+E46+G46,0)</f>
-        <v>3588.0</v>
+        <v/>
       </c>
       <c r="G46" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H46" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B46,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B46+1))</f>
-        <v>1228.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B46,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B46+1))</f>
+        <v/>
       </c>
       <c r="I46" s="274">
         <f>IFERROR(F46-H46,0)</f>
-        <v>2360.0</v>
+        <v/>
       </c>
       <c r="J46" s="275">
         <f>IFERROR(I46/F46,0)</f>
-        <v>0.657748</v>
+        <v/>
       </c>
       <c r="K46" s="250" t="n"/>
       <c r="L46" s="276" t="inlineStr">
@@ -11661,22 +11661,22 @@
       </c>
       <c r="F47" s="50">
         <f>IFERROR(D47+E47+G47,0)</f>
-        <v>4477.0</v>
+        <v/>
       </c>
       <c r="G47" s="257" t="n">
         <v>165</v>
       </c>
       <c r="H47" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B47,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B47+1))</f>
-        <v>1945.53</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B47,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B47+1))</f>
+        <v/>
       </c>
       <c r="I47" s="259">
         <f>IFERROR(F47-H47,0)</f>
-        <v>2531.47</v>
+        <v/>
       </c>
       <c r="J47" s="260">
         <f>IFERROR(I47/F47,0)</f>
-        <v>0.565439</v>
+        <v/>
       </c>
       <c r="K47" s="254" t="n"/>
       <c r="L47" s="261" t="inlineStr">
@@ -11721,22 +11721,22 @@
       </c>
       <c r="F48" s="38">
         <f>IFERROR(D48+E48+G48,0)</f>
-        <v>2029.0</v>
+        <v/>
       </c>
       <c r="G48" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H48" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B48,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B48+1))</f>
-        <v>5250.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B48,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B48+1))</f>
+        <v/>
       </c>
       <c r="I48" s="274">
         <f>IFERROR(F48-H48,0)</f>
-        <v>-3221.0</v>
+        <v/>
       </c>
       <c r="J48" s="275">
         <f>IFERROR(I48/F48,0)</f>
-        <v>-1.587482</v>
+        <v/>
       </c>
       <c r="K48" s="250" t="n"/>
       <c r="L48" s="276" t="inlineStr">
@@ -11781,22 +11781,22 @@
       </c>
       <c r="F49" s="50">
         <f>IFERROR(D49+E49+G49,0)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="G49" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H49" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B49,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B49+1))</f>
-        <v>3865.06</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B49,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B49+1))</f>
+        <v/>
       </c>
       <c r="I49" s="259">
         <f>IFERROR(F49-H49,0)</f>
-        <v>-3865.06</v>
+        <v/>
       </c>
       <c r="J49" s="260">
         <f>IFERROR(I49/F49,0)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K49" s="254" t="n"/>
       <c r="L49" s="261" t="inlineStr">
@@ -11841,22 +11841,22 @@
       </c>
       <c r="F50" s="38">
         <f>IFERROR(D50+E50+G50,0)</f>
-        <v>3389.0</v>
+        <v/>
       </c>
       <c r="G50" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H50" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B50,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B50+1))</f>
-        <v>2683.27</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B50,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B50+1))</f>
+        <v/>
       </c>
       <c r="I50" s="274">
         <f>IFERROR(F50-H50,0)</f>
-        <v>705.73</v>
+        <v/>
       </c>
       <c r="J50" s="275">
         <f>IFERROR(I50/F50,0)</f>
-        <v>0.208241</v>
+        <v/>
       </c>
       <c r="K50" s="250" t="n"/>
       <c r="L50" s="276" t="inlineStr">
@@ -11901,22 +11901,22 @@
       </c>
       <c r="F51" s="50">
         <f>IFERROR(D51+E51+G51,0)</f>
-        <v>4133.0</v>
+        <v/>
       </c>
       <c r="G51" s="257" t="n">
         <v>55</v>
       </c>
       <c r="H51" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B51,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B51+1))</f>
-        <v>1581.27</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B51,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B51+1))</f>
+        <v/>
       </c>
       <c r="I51" s="259">
         <f>IFERROR(F51-H51,0)</f>
-        <v>2551.73</v>
+        <v/>
       </c>
       <c r="J51" s="260">
         <f>IFERROR(I51/F51,0)</f>
-        <v>0.617404</v>
+        <v/>
       </c>
       <c r="K51" s="254" t="n"/>
       <c r="L51" s="261" t="inlineStr">
@@ -11961,22 +11961,22 @@
       </c>
       <c r="F52" s="38">
         <f>IFERROR(D52+E52+G52,0)</f>
-        <v>4522.0</v>
+        <v/>
       </c>
       <c r="G52" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H52" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B52,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B52+1))</f>
-        <v>2341.23</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B52,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B52+1))</f>
+        <v/>
       </c>
       <c r="I52" s="274">
         <f>IFERROR(F52-H52,0)</f>
-        <v>2180.77</v>
+        <v/>
       </c>
       <c r="J52" s="275">
         <f>IFERROR(I52/F52,0)</f>
-        <v>0.482258</v>
+        <v/>
       </c>
       <c r="K52" s="250" t="n"/>
       <c r="L52" s="276" t="inlineStr">
@@ -12021,22 +12021,22 @@
       </c>
       <c r="F53" s="50">
         <f>IFERROR(D53+E53+G53,0)</f>
-        <v>3108.0</v>
+        <v/>
       </c>
       <c r="G53" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H53" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B53,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B53+1))</f>
-        <v>318.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B53,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B53+1))</f>
+        <v/>
       </c>
       <c r="I53" s="259">
         <f>IFERROR(F53-H53,0)</f>
-        <v>2790.0</v>
+        <v/>
       </c>
       <c r="J53" s="260">
         <f>IFERROR(I53/F53,0)</f>
-        <v>0.897683</v>
+        <v/>
       </c>
       <c r="K53" s="254" t="inlineStr">
         <is>
@@ -12085,22 +12085,22 @@
       </c>
       <c r="F54" s="38">
         <f>IFERROR(D54+E54+G54,0)</f>
-        <v>6077.0</v>
+        <v/>
       </c>
       <c r="G54" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H54" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B54,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B54+1))</f>
-        <v>2809.6</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B54,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B54+1))</f>
+        <v/>
       </c>
       <c r="I54" s="274">
         <f>IFERROR(F54-H54,0)</f>
-        <v>3267.4</v>
+        <v/>
       </c>
       <c r="J54" s="275">
         <f>IFERROR(I54/F54,0)</f>
-        <v>0.537667</v>
+        <v/>
       </c>
       <c r="K54" s="250" t="inlineStr">
         <is>
@@ -12149,22 +12149,22 @@
       </c>
       <c r="F55" s="50">
         <f>IFERROR(D55+E55+G55,0)</f>
-        <v>2634.0</v>
+        <v/>
       </c>
       <c r="G55" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H55" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B55,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B55+1))</f>
-        <v>6877.73</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B55,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B55+1))</f>
+        <v/>
       </c>
       <c r="I55" s="259">
         <f>IFERROR(F55-H55,0)</f>
-        <v>-4243.73</v>
+        <v/>
       </c>
       <c r="J55" s="260">
         <f>IFERROR(I55/F55,0)</f>
-        <v>-1.611135</v>
+        <v/>
       </c>
       <c r="K55" s="254" t="n"/>
       <c r="L55" s="261" t="inlineStr">
@@ -12209,22 +12209,22 @@
       </c>
       <c r="F56" s="38">
         <f>IFERROR(D56+E56+G56,0)</f>
-        <v>3690.0</v>
+        <v/>
       </c>
       <c r="G56" s="272" t="n">
         <v>0</v>
       </c>
       <c r="H56" s="273">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B56,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B56+1))</f>
-        <v>4200.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B56,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B56+1))</f>
+        <v/>
       </c>
       <c r="I56" s="274">
         <f>IFERROR(F56-H56,0)</f>
-        <v>-510.0</v>
+        <v/>
       </c>
       <c r="J56" s="275">
         <f>IFERROR(I56/F56,0)</f>
-        <v>-0.138211</v>
+        <v/>
       </c>
       <c r="K56" s="250" t="n"/>
       <c r="L56" s="276" t="inlineStr">
@@ -12269,22 +12269,22 @@
       </c>
       <c r="F57" s="50">
         <f>IFERROR(D57+E57+G57,0)</f>
-        <v>3660.0</v>
+        <v/>
       </c>
       <c r="G57" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H57" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B57,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B57+1))</f>
-        <v>49.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B57,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B57+1))</f>
+        <v/>
       </c>
       <c r="I57" s="259">
         <f>IFERROR(F57-H57,0)</f>
-        <v>3611.0</v>
+        <v/>
       </c>
       <c r="J57" s="260">
         <f>IFERROR(I57/F57,0)</f>
-        <v>0.986612</v>
+        <v/>
       </c>
       <c r="K57" s="254" t="n"/>
       <c r="L57" s="261" t="inlineStr">
@@ -12329,22 +12329,22 @@
       </c>
       <c r="F58" s="50">
         <f>IFERROR(D58+E58+G58+U58,0)</f>
-        <v>3688.0</v>
+        <v/>
       </c>
       <c r="G58" s="257" t="n">
         <v>195</v>
       </c>
       <c r="H58" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B58,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B58+1))</f>
-        <v>1415.43</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B58,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B58+1))</f>
+        <v/>
       </c>
       <c r="I58" s="259">
         <f>IFERROR(F58-H58,0)</f>
-        <v>2272.57</v>
+        <v/>
       </c>
       <c r="J58" s="260">
         <f>IFERROR(I58/F58,0)</f>
-        <v>0.616207</v>
+        <v/>
       </c>
       <c r="K58" s="254" t="n"/>
       <c r="L58" s="261" t="inlineStr">
@@ -12393,22 +12393,22 @@
       </c>
       <c r="F59" s="50">
         <f>IFERROR(D59+E59+G59+U59,0)</f>
-        <v>6015.0</v>
+        <v/>
       </c>
       <c r="G59" s="257" t="n">
         <v>120</v>
       </c>
       <c r="H59" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B59,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B59+1))</f>
-        <v>1820.89</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B59,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B59+1))</f>
+        <v/>
       </c>
       <c r="I59" s="259">
         <f>IFERROR(F59-H59,0)</f>
-        <v>4194.11</v>
+        <v/>
       </c>
       <c r="J59" s="260">
         <f>IFERROR(I59/F59,0)</f>
-        <v>0.697275</v>
+        <v/>
       </c>
       <c r="K59" s="254" t="n"/>
       <c r="L59" s="261" t="inlineStr">
@@ -12457,22 +12457,22 @@
       </c>
       <c r="F60" s="50">
         <f>IFERROR(D60+E60+G60+U60,0)</f>
-        <v>3500.0</v>
+        <v/>
       </c>
       <c r="G60" s="257" t="n">
         <v>70</v>
       </c>
       <c r="H60" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B60,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B60+1))</f>
-        <v>2094.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B60,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B60+1))</f>
+        <v/>
       </c>
       <c r="I60" s="259">
         <f>IFERROR(F60-H60,0)</f>
-        <v>1406.0</v>
+        <v/>
       </c>
       <c r="J60" s="260">
         <f>IFERROR(I60/F60,0)</f>
-        <v>0.401714</v>
+        <v/>
       </c>
       <c r="K60" s="254" t="n"/>
       <c r="L60" s="261" t="inlineStr">
@@ -12521,22 +12521,22 @@
       </c>
       <c r="F61" s="50">
         <f>IFERROR(D61+E61+G61+U61,0)</f>
-        <v>2725.0</v>
+        <v/>
       </c>
       <c r="G61" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H61" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B61,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B61+1))</f>
-        <v>10207.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B61,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B61+1))</f>
+        <v/>
       </c>
       <c r="I61" s="259">
         <f>IFERROR(F61-H61,0)</f>
-        <v>-7482.0</v>
+        <v/>
       </c>
       <c r="J61" s="260">
         <f>IFERROR(I61/F61,0)</f>
-        <v>-2.745688</v>
+        <v/>
       </c>
       <c r="K61" s="254" t="n"/>
       <c r="L61" s="261" t="inlineStr">
@@ -12585,22 +12585,22 @@
       </c>
       <c r="F62" s="50">
         <f>IFERROR(D62+E62+G62+U62+Y62,0)</f>
-        <v>3990.0</v>
+        <v/>
       </c>
       <c r="G62" s="257" t="n">
         <v>120</v>
       </c>
       <c r="H62" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B62,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B62+1))</f>
-        <v>3142.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B62,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B62+1))</f>
+        <v/>
       </c>
       <c r="I62" s="259">
         <f>IFERROR(F62-H62,0)</f>
-        <v>848.0</v>
+        <v/>
       </c>
       <c r="J62" s="260">
         <f>IFERROR(I62/F62,0)</f>
-        <v>0.212531</v>
+        <v/>
       </c>
       <c r="K62" s="254" t="n"/>
       <c r="L62" s="261" t="inlineStr">
@@ -12653,22 +12653,22 @@
       </c>
       <c r="F63" s="50">
         <f>IFERROR(D63+E63+G63+U63+Y63,0)</f>
-        <v>3915.0</v>
+        <v/>
       </c>
       <c r="G63" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H63" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B63,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B63+1))</f>
-        <v>596.38</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B63,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B63+1))</f>
+        <v/>
       </c>
       <c r="I63" s="259">
         <f>IFERROR(F63-H63,0)</f>
-        <v>3318.62</v>
+        <v/>
       </c>
       <c r="J63" s="260">
         <f>IFERROR(I63/F63,0)</f>
-        <v>0.847668</v>
+        <v/>
       </c>
       <c r="K63" s="254" t="n"/>
       <c r="L63" s="261" t="inlineStr">
@@ -12721,22 +12721,22 @@
       </c>
       <c r="F64" s="50">
         <f>IFERROR(D64+E64+G64+U64+Y64,0)</f>
-        <v>5565.0</v>
+        <v/>
       </c>
       <c r="G64" s="257" t="n">
         <v>130</v>
       </c>
       <c r="H64" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B64,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B64+1))</f>
-        <v>2606.86</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B64,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B64+1))</f>
+        <v/>
       </c>
       <c r="I64" s="259">
         <f>IFERROR(F64-H64,0)</f>
-        <v>2958.14</v>
+        <v/>
       </c>
       <c r="J64" s="260">
         <f>IFERROR(I64/F64,0)</f>
-        <v>0.531562</v>
+        <v/>
       </c>
       <c r="K64" s="254" t="n"/>
       <c r="L64" s="261" t="inlineStr">
@@ -12789,22 +12789,22 @@
       </c>
       <c r="F65" s="50">
         <f>IFERROR(D65+E65+G65+U65+Y65,0)</f>
-        <v>12495.0</v>
+        <v/>
       </c>
       <c r="G65" s="257" t="n">
         <v>2385</v>
       </c>
       <c r="H65" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B65,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B65+1))</f>
-        <v>1657.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B65,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B65+1))</f>
+        <v/>
       </c>
       <c r="I65" s="259">
         <f>IFERROR(F65-H65,0)</f>
-        <v>10838.0</v>
+        <v/>
       </c>
       <c r="J65" s="260">
         <f>IFERROR(I65/F65,0)</f>
-        <v>0.867387</v>
+        <v/>
       </c>
       <c r="K65" s="254" t="n"/>
       <c r="L65" s="261" t="inlineStr">
@@ -12857,22 +12857,22 @@
       </c>
       <c r="F66" s="50">
         <f>IFERROR(D66+E66+G66+U66+Y66,0)</f>
-        <v>2622.0</v>
+        <v/>
       </c>
       <c r="G66" s="257" t="n">
         <v>300</v>
       </c>
       <c r="H66" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B66,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B66+1))</f>
-        <v>1951.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B66,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B66+1))</f>
+        <v/>
       </c>
       <c r="I66" s="259">
         <f>IFERROR(F66-H66,0)</f>
-        <v>671.0</v>
+        <v/>
       </c>
       <c r="J66" s="260">
         <f>IFERROR(I66/F66,0)</f>
-        <v>0.255912</v>
+        <v/>
       </c>
       <c r="K66" s="254" t="n"/>
       <c r="L66" s="261" t="inlineStr">
@@ -12925,22 +12925,22 @@
       </c>
       <c r="F67" s="50">
         <f>IFERROR(D67+E67+G67+U67+Y67,0)</f>
-        <v>2900.0</v>
+        <v/>
       </c>
       <c r="G67" s="257" t="n">
         <v>290</v>
       </c>
       <c r="H67" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B67,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B67+1))</f>
-        <v>5250.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B67,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B67+1))</f>
+        <v/>
       </c>
       <c r="I67" s="259">
         <f>IFERROR(F67-H67,0)</f>
-        <v>-2350.0</v>
+        <v/>
       </c>
       <c r="J67" s="260">
         <f>IFERROR(I67/F67,0)</f>
-        <v>-0.810345</v>
+        <v/>
       </c>
       <c r="K67" s="254" t="n"/>
       <c r="L67" s="261" t="inlineStr">
@@ -12993,22 +12993,22 @@
       </c>
       <c r="F68" s="50">
         <f>IFERROR(D68+E68+G68+U68+Y68,0)</f>
-        <v>4955.0</v>
+        <v/>
       </c>
       <c r="G68" s="257" t="n">
         <v>0</v>
       </c>
       <c r="H68" s="258">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;B68,'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;(B68+1))</f>
-        <v>2459.0</v>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B68,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B68+1))</f>
+        <v/>
       </c>
       <c r="I68" s="259">
         <f>IFERROR(F68-H68,0)</f>
-        <v>2496.0</v>
+        <v/>
       </c>
       <c r="J68" s="260">
         <f>IFERROR(I68/F68,0)</f>
-        <v>0.503734</v>
+        <v/>
       </c>
       <c r="K68" s="254" t="n"/>
       <c r="L68" s="261" t="inlineStr">
@@ -21862,9 +21862,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -21927,6 +21927,7 @@
     <row r="3">
       <c r="A3" s="401" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="59" t="inlineStr">
         <is>
@@ -21971,35 +21972,35 @@
     </row>
     <row r="6" ht="15.6" customHeight="1" s="313">
       <c r="B6" s="60">
-        <f>SUMIFS($F$8:$F$500,$B$8:$B$500,TODAY())</f>
+        <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,TODAY())</f>
         <v/>
       </c>
       <c r="C6" s="61">
-        <f>SUMIFS($F$8:$F$500,$B$8:$B$500,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$500,"&lt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+7))</f>
+        <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+7))</f>
         <v/>
       </c>
       <c r="D6" s="62">
-        <f>SUMIFS($F$8:$F$500,$B$8:$B$500,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$500,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
+        <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
         <v/>
       </c>
       <c r="E6" s="61">
-        <f>SUMIF($E$8:$E$500,"Ingredients*",$F$8:$F$500)</f>
+        <f>SUMIF($E$8:$E$5000,"Ingredients*",$F$8:$F$5000)</f>
         <v/>
       </c>
       <c r="F6" s="63">
-        <f>SUMIF($E$8:$E$500,"Staff*",$F$8:$F$500)</f>
+        <f>SUMIF($E$8:$E$5000,"Staff*",$F$8:$F$5000)</f>
         <v/>
       </c>
       <c r="G6" s="62">
-        <f>SUMIF($E$8:$E$500,"Supplies*",$F$8:$F$500)+SUMIF($E$8:$E$500,"Utilities*",$F$8:$F$500)</f>
+        <f>SUMIF($E$8:$E$5000,"Supplies*",$F$8:$F$5000)+SUMIF($E$8:$E$5000,"Utilities*",$F$8:$F$5000)</f>
         <v/>
       </c>
       <c r="H6" s="60">
-        <f>SUMIFS($F$8:$F$500,$B$8:$B$500,TODAY())</f>
+        <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,TODAY())</f>
         <v/>
       </c>
       <c r="I6" s="60">
-        <f>SUMIFS($F$8:$F$500,$B$8:$B$500,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$500,"&lt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+7))</f>
+        <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+7))</f>
         <v/>
       </c>
     </row>
@@ -43399,23 +43400,23 @@
     </row>
     <row r="6" ht="25.5" customHeight="1" s="313">
       <c r="B6" s="79">
-        <f>COUNTA(B9:B200)</f>
+        <f>COUNTA(B9:B2000)</f>
         <v/>
       </c>
       <c r="D6" s="80">
-        <f>COUNTIF(J9:J200,"⚠️ LOW STOCK")</f>
+        <f>COUNTIF(J9:J2000,"⚠️ LOW STOCK")</f>
         <v/>
       </c>
       <c r="E6" s="80">
-        <f>COUNTIF(J9:J200,"⚠️ LOW STOCK")+COUNTIF(J9:J200,"🚫 OUT OF STOCK")</f>
+        <f>COUNTIF(J9:J2000,"⚠️ LOW STOCK")+COUNTIF(J9:J2000,"🚫 OUT OF STOCK")</f>
         <v/>
       </c>
       <c r="F6" s="81">
-        <f>COUNTIF(J9:J200,"🚫 OUT OF STOCK")</f>
+        <f>COUNTIF(J9:J2000,"🚫 OUT OF STOCK")</f>
         <v/>
       </c>
       <c r="H6" s="81">
-        <f>COUNTIF(J9:J200,"⚠️ LOW STOCK")+COUNTIF(J9:J200,"🚫 OUT OF STOCK")</f>
+        <f>COUNTIF(J9:J2000,"⚠️ LOW STOCK")+COUNTIF(J9:J2000,"🚫 OUT OF STOCK")</f>
         <v/>
       </c>
       <c r="J6" s="82">
@@ -48970,31 +48971,31 @@
     </row>
     <row r="6" ht="25.5" customHeight="1" s="313">
       <c r="B6" s="79">
-        <f>COUNTA(C9:C308)-1</f>
+        <f>COUNTA(C9:C3000)-1</f>
         <v/>
       </c>
       <c r="C6" s="121">
-        <f>COUNTIF(K9:K308,"Pending")</f>
+        <f>COUNTIF(K9:K3000,"Pending")</f>
         <v/>
       </c>
       <c r="D6" s="122">
-        <f>COUNTIF(K9:K308,"In Transit")</f>
+        <f>COUNTIF(K9:K3000,"In Transit")</f>
         <v/>
       </c>
       <c r="E6" s="123">
-        <f>COUNTIF(K9:K308,"Received")</f>
+        <f>COUNTIF(K9:K3000,"Received")</f>
         <v/>
       </c>
       <c r="F6" s="124">
-        <f>SUMIF(K9:K308,"Received",J9:J308)</f>
+        <f>SUMIF(K9:K3000,"Received",J9:J3000)</f>
         <v/>
       </c>
       <c r="G6" s="61">
-        <f>SUMIF(K9:K308,"Pending",J9:J308)</f>
+        <f>SUMIF(K9:K3000,"Pending",J9:J3000)</f>
         <v/>
       </c>
       <c r="H6" s="121">
-        <f>COUNTIF(K9:K308,"Pending")+COUNTIF(K9:K308,"In Transit")</f>
+        <f>COUNTIF(K9:K3000,"Pending")+COUNTIF(K9:K3000,"In Transit")</f>
         <v/>
       </c>
     </row>
@@ -52986,15 +52987,15 @@
         </is>
       </c>
       <c r="B4" s="413">
-        <f>SUMIFS('📅 Daily Log'!$F$8:$F$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$F$8:$F$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C4" s="413">
-        <f>SUMIFS('📅 Daily Log'!$F$8:$F$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$F$8:$F$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D4" s="413">
-        <f>SUMIFS('📅 Daily Log'!$F$8:$F$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$F$8:$F$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E4" s="409" t="n"/>
@@ -53013,15 +53014,15 @@
         </is>
       </c>
       <c r="B5" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C5" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D5" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E5" s="409" t="n"/>
@@ -53067,15 +53068,15 @@
         </is>
       </c>
       <c r="B7" s="416">
-        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$500,"&gt;0",'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$5000,"&gt;0",'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C7" s="416">
-        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$500,"&gt;0",'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$5000,"&gt;0",'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D7" s="416">
-        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$500,"&gt;0",'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$5000,"&gt;0",'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E7" s="409" t="n"/>
@@ -53165,15 +53166,15 @@
         </is>
       </c>
       <c r="B11" s="413">
-        <f>SUMIFS('📅 Daily Log'!$D$8:$D$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$D$8:$D$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C11" s="413">
-        <f>SUMIFS('📅 Daily Log'!$D$8:$D$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$D$8:$D$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D11" s="413">
-        <f>SUMIFS('📅 Daily Log'!$D$8:$D$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$D$8:$D$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E11" s="409" t="n"/>
@@ -53192,15 +53193,15 @@
         </is>
       </c>
       <c r="B12" s="413">
-        <f>SUMIFS('📅 Daily Log'!$E$8:$E$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$E$8:$E$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C12" s="413">
-        <f>SUMIFS('📅 Daily Log'!$E$8:$E$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$E$8:$E$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D12" s="413">
-        <f>SUMIFS('📅 Daily Log'!$E$8:$E$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$E$8:$E$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E12" s="409" t="n"/>
@@ -53219,15 +53220,15 @@
         </is>
       </c>
       <c r="B13" s="413">
-        <f>SUMIFS('📅 Daily Log'!$G$8:$G$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$G$8:$G$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C13" s="413">
-        <f>SUMIFS('📅 Daily Log'!$G$8:$G$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$G$8:$G$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D13" s="413">
-        <f>SUMIFS('📅 Daily Log'!$G$8:$G$500,'📅 Daily Log'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('📅 Daily Log'!$G$8:$G$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E13" s="409" t="n"/>
@@ -53317,15 +53318,15 @@
         </is>
       </c>
       <c r="B17" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A17,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A17,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C17" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A17,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A17,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D17" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A17,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A17,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E17" s="409" t="n"/>
@@ -53344,15 +53345,15 @@
         </is>
       </c>
       <c r="B18" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A18,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A18,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C18" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A18,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A18,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D18" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A18,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A18,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E18" s="409" t="n"/>
@@ -53371,15 +53372,15 @@
         </is>
       </c>
       <c r="B19" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A19,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A19,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C19" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A19,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A19,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D19" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A19,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A19,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E19" s="409" t="n"/>
@@ -53398,15 +53399,15 @@
         </is>
       </c>
       <c r="B20" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A20,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A20,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C20" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A20,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A20,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D20" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A20,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A20,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E20" s="409" t="n"/>
@@ -53425,15 +53426,15 @@
         </is>
       </c>
       <c r="B21" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A21,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A21,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C21" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A21,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A21,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D21" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A21,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A21,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E21" s="409" t="n"/>
@@ -53452,15 +53453,15 @@
         </is>
       </c>
       <c r="B22" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A22,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A22,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C22" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A22,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A22,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D22" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A22,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A22,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E22" s="409" t="n"/>
@@ -53479,15 +53480,15 @@
         </is>
       </c>
       <c r="B23" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A23,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A23,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C23" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A23,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A23,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D23" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A23,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A23,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E23" s="409" t="n"/>
@@ -53506,15 +53507,15 @@
         </is>
       </c>
       <c r="B24" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A24,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A24,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C24" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A24,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A24,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D24" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A24,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A24,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E24" s="409" t="n"/>
@@ -53533,15 +53534,15 @@
         </is>
       </c>
       <c r="B25" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A25,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A25,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C25" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A25,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A25,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D25" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A25,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A25,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E25" s="409" t="n"/>
@@ -53560,15 +53561,15 @@
         </is>
       </c>
       <c r="B26" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A26,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A26,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C26" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A26,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A26,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D26" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A26,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A26,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E26" s="409" t="n"/>
@@ -53587,15 +53588,15 @@
         </is>
       </c>
       <c r="B27" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A27,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A27,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C27" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A27,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A27,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D27" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A27,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A27,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E27" s="409" t="n"/>
@@ -53614,15 +53615,15 @@
         </is>
       </c>
       <c r="B28" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A28,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A28,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C28" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A28,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A28,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D28" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A28,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A28,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E28" s="409" t="n"/>
@@ -53641,15 +53642,15 @@
         </is>
       </c>
       <c r="B29" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A29,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A29,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C29" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A29,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A29,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D29" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A29,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A29,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E29" s="409" t="n"/>
@@ -53668,15 +53669,15 @@
         </is>
       </c>
       <c r="B30" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A30,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A30,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C30" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A30,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A30,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D30" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A30,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A30,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E30" s="409" t="n"/>
@@ -53695,15 +53696,15 @@
         </is>
       </c>
       <c r="B31" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A31,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A31,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C31" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A31,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A31,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D31" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A31,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A31,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E31" s="409" t="n"/>
@@ -53722,15 +53723,15 @@
         </is>
       </c>
       <c r="B32" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A32,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A32,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C32" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A32,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A32,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D32" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A32,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A32,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E32" s="409" t="n"/>
@@ -53749,15 +53750,15 @@
         </is>
       </c>
       <c r="B33" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A33,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A33,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C33" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A33,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A33,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D33" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A33,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A33,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E33" s="409" t="n"/>
@@ -53776,15 +53777,15 @@
         </is>
       </c>
       <c r="B34" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A34,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A34,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C34" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A34,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A34,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D34" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A34,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A34,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E34" s="409" t="n"/>
@@ -53803,15 +53804,15 @@
         </is>
       </c>
       <c r="B35" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A35,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A35,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C35" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A35,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A35,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D35" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A35,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A35,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E35" s="409" t="n"/>
@@ -53830,15 +53831,15 @@
         </is>
       </c>
       <c r="B36" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A36,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A36,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C36" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A36,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A36,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D36" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A36,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A36,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E36" s="409" t="n"/>
@@ -53857,15 +53858,15 @@
         </is>
       </c>
       <c r="B37" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A37,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A37,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C37" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A37,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A37,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D37" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A37,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A37,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E37" s="409" t="n"/>
@@ -53884,15 +53885,15 @@
         </is>
       </c>
       <c r="B38" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A38,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A38,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C38" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A38,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A38,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D38" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A38,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A38,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E38" s="409" t="n"/>
@@ -53911,15 +53912,15 @@
         </is>
       </c>
       <c r="B39" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A39,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A39,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C39" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A39,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A39,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D39" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A39,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A39,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E39" s="409" t="n"/>
@@ -53938,15 +53939,15 @@
         </is>
       </c>
       <c r="B40" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A40,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A40,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C40" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A40,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A40,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D40" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A40,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A40,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E40" s="409" t="n"/>
@@ -53965,15 +53966,15 @@
         </is>
       </c>
       <c r="B41" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A41,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C41" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A41,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D41" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A41,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E41" s="409" t="n"/>
@@ -53992,15 +53993,15 @@
         </is>
       </c>
       <c r="B42" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A42,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A42,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C42" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A42,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A42,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D42" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A42,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A42,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E42" s="409" t="n"/>
@@ -54019,15 +54020,15 @@
         </is>
       </c>
       <c r="B43" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A43,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A43,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C43" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A43,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A43,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D43" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A43,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A43,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E43" s="409" t="n"/>
@@ -54046,15 +54047,15 @@
         </is>
       </c>
       <c r="B44" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A44,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A44,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C44" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A44,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A44,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D44" s="413">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$E$8:$E$500,$A44,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A44,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E44" s="409" t="n"/>
@@ -54073,15 +54074,15 @@
         </is>
       </c>
       <c r="B45" s="414">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,6,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C45" s="414">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,7,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D45" s="414">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$500,'💸 Expenses'!$B$8:$B$500,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$500,"&lt;"&amp;DATE(2026,8,1))</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E45" s="409" t="n"/>

</xml_diff>

<commit_message>
updated rent and ec bill
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -19,7 +19,7 @@
     <sheet name="💰 Owner Ledger" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -1008,7 +1008,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1358,11 +1358,15 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25"/>
   </cellStyleXfs>
-  <cellXfs count="441">
+  <cellXfs count="443">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -2486,6 +2490,10 @@
     <xf numFmtId="3" fontId="99" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="100" fillId="58" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5482,11 +5490,11 @@
         </is>
       </c>
       <c r="C147" s="268" t="n">
-        <v>16727.81</v>
+        <v>42716.85</v>
       </c>
       <c r="E147" s="286" t="inlineStr">
         <is>
-          <t>Advance from capital-funded operating costs; repaid from operating cash: $20,000 (21-Jul) + $2,587 (22-Jul). Net advance still owed = $16,727.81.</t>
+          <t>Operating costs funded from partner capital, net of repayments. Latest addition 04-Aug-2026 $25,989.04. Still owed by Operations: $42,716.85.</t>
         </is>
       </c>
     </row>
@@ -22765,8 +22773,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -22790,7 +22798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J576"/>
+  <dimension ref="A1:J578"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -47061,6 +47069,92 @@
       <c r="J576" s="423" t="inlineStr">
         <is>
           <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="B577" s="429" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C577" s="297" t="inlineStr">
+        <is>
+          <t>Renta mensual Agosto 2026</t>
+        </is>
+      </c>
+      <c r="D577" s="298" t="inlineStr">
+        <is>
+          <t>Arrendador</t>
+        </is>
+      </c>
+      <c r="E577" s="297" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="F577" s="299" t="n">
+        <v>17200.04</v>
+      </c>
+      <c r="G577" s="300" t="inlineStr">
+        <is>
+          <t>Capital</t>
+        </is>
+      </c>
+      <c r="H577" s="300" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="I577" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J577" s="423" t="inlineStr">
+        <is>
+          <t>Renta contractual 19,066.68/mes. Jun y Jul se pagaron 20,000 c/u = sobrepago 933.32 x2 = 1,866.64, acreditado este mes: 19,066.68 - 1,866.64 = 17,200.04. Pagado con capital de socios. DESDE SEPTIEMBRE la renta mensual es 19,066.68.</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="B578" s="429" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C578" s="297" t="inlineStr">
+        <is>
+          <t>Recibo de luz CFE</t>
+        </is>
+      </c>
+      <c r="D578" s="298" t="inlineStr">
+        <is>
+          <t>CFE</t>
+        </is>
+      </c>
+      <c r="E578" s="297" t="inlineStr">
+        <is>
+          <t>Utilities/Electricity</t>
+        </is>
+      </c>
+      <c r="F578" s="299" t="n">
+        <v>8789</v>
+      </c>
+      <c r="G578" s="300" t="inlineStr">
+        <is>
+          <t>Capital</t>
+        </is>
+      </c>
+      <c r="H578" s="300" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="I578" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J578" s="423" t="inlineStr">
+        <is>
+          <t>Recibo de luz pagado con capital de socios.</t>
         </is>
       </c>
     </row>
@@ -50977,7 +51071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="18.33203125" customWidth="1" style="331" min="1" max="1"/>
@@ -52637,61 +52731,405 @@
       <c r="D92" s="264" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="262" t="n"/>
-      <c r="B93" s="262" t="inlineStr">
-        <is>
-          <t>TOTAL TIPS PASSED THROUGH</t>
-        </is>
-      </c>
+      <c r="A93" s="263" t="n"/>
+      <c r="B93" s="262" t="n"/>
       <c r="C93" s="262" t="n"/>
-      <c r="D93" s="264">
-        <f>SUM(D63:D92)</f>
-        <v/>
-      </c>
+      <c r="D93" s="264" t="n"/>
+      <c r="E93" s="423" t="n"/>
+      <c r="F93" s="423" t="n"/>
+      <c r="G93" s="423" t="n"/>
+      <c r="H93" s="423" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="262" t="inlineStr">
-        <is>
-          <t>Customer tips collected &amp; handed to staff. Excluded from P&amp;L — nets to zero (received = paid).</t>
-        </is>
-      </c>
+      <c r="A94" s="263" t="n"/>
       <c r="B94" s="262" t="n"/>
       <c r="C94" s="262" t="n"/>
-      <c r="D94" s="262" t="n"/>
+      <c r="D94" s="264" t="n"/>
+      <c r="E94" s="423" t="n"/>
+      <c r="F94" s="423" t="n"/>
+      <c r="G94" s="423" t="n"/>
+      <c r="H94" s="423" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="263" t="n"/>
+      <c r="B95" s="262" t="n"/>
+      <c r="C95" s="262" t="n"/>
+      <c r="D95" s="264" t="n"/>
+      <c r="E95" s="423" t="n"/>
+      <c r="F95" s="423" t="n"/>
+      <c r="G95" s="423" t="n"/>
+      <c r="H95" s="423" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="263" t="n"/>
+      <c r="B96" s="262" t="n"/>
+      <c r="C96" s="262" t="n"/>
+      <c r="D96" s="264" t="n"/>
+      <c r="E96" s="423" t="n"/>
+      <c r="F96" s="423" t="n"/>
+      <c r="G96" s="423" t="n"/>
+      <c r="H96" s="423" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="263" t="n"/>
+      <c r="B97" s="262" t="n"/>
+      <c r="C97" s="262" t="n"/>
+      <c r="D97" s="264" t="n"/>
+      <c r="E97" s="423" t="n"/>
+      <c r="F97" s="423" t="n"/>
+      <c r="G97" s="423" t="n"/>
+      <c r="H97" s="423" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="263" t="n"/>
+      <c r="B98" s="262" t="n"/>
+      <c r="C98" s="262" t="n"/>
+      <c r="D98" s="264" t="n"/>
+      <c r="E98" s="423" t="n"/>
+      <c r="F98" s="423" t="n"/>
+      <c r="G98" s="423" t="n"/>
+      <c r="H98" s="423" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="263" t="n"/>
+      <c r="B99" s="262" t="n"/>
+      <c r="C99" s="262" t="n"/>
+      <c r="D99" s="264" t="n"/>
+      <c r="E99" s="423" t="n"/>
+      <c r="F99" s="423" t="n"/>
+      <c r="G99" s="423" t="n"/>
+      <c r="H99" s="423" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="263" t="n"/>
+      <c r="B100" s="262" t="n"/>
+      <c r="C100" s="262" t="n"/>
+      <c r="D100" s="264" t="n"/>
+      <c r="E100" s="423" t="n"/>
+      <c r="F100" s="423" t="n"/>
+      <c r="G100" s="423" t="n"/>
+      <c r="H100" s="423" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="263" t="n"/>
+      <c r="B101" s="262" t="n"/>
+      <c r="C101" s="262" t="n"/>
+      <c r="D101" s="264" t="n"/>
+      <c r="E101" s="423" t="n"/>
+      <c r="F101" s="423" t="n"/>
+      <c r="G101" s="423" t="n"/>
+      <c r="H101" s="423" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="263" t="n"/>
+      <c r="B102" s="262" t="n"/>
+      <c r="C102" s="262" t="n"/>
+      <c r="D102" s="264" t="n"/>
+      <c r="E102" s="423" t="n"/>
+      <c r="F102" s="423" t="n"/>
+      <c r="G102" s="423" t="n"/>
+      <c r="H102" s="423" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="263" t="n"/>
+      <c r="B103" s="262" t="n"/>
+      <c r="C103" s="262" t="n"/>
+      <c r="D103" s="264" t="n"/>
+      <c r="E103" s="423" t="n"/>
+      <c r="F103" s="423" t="n"/>
+      <c r="G103" s="423" t="n"/>
+      <c r="H103" s="423" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="263" t="n"/>
+      <c r="B104" s="262" t="n"/>
+      <c r="C104" s="262" t="n"/>
+      <c r="D104" s="264" t="n"/>
+      <c r="E104" s="423" t="n"/>
+      <c r="F104" s="423" t="n"/>
+      <c r="G104" s="423" t="n"/>
+      <c r="H104" s="423" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="263" t="n"/>
+      <c r="B105" s="262" t="n"/>
+      <c r="C105" s="262" t="n"/>
+      <c r="D105" s="264" t="n"/>
+      <c r="E105" s="423" t="n"/>
+      <c r="F105" s="423" t="n"/>
+      <c r="G105" s="423" t="n"/>
+      <c r="H105" s="423" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="263" t="n"/>
+      <c r="B106" s="262" t="n"/>
+      <c r="C106" s="262" t="n"/>
+      <c r="D106" s="264" t="n"/>
+      <c r="E106" s="423" t="n"/>
+      <c r="F106" s="423" t="n"/>
+      <c r="G106" s="423" t="n"/>
+      <c r="H106" s="423" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="263" t="n"/>
+      <c r="B107" s="262" t="n"/>
+      <c r="C107" s="262" t="n"/>
+      <c r="D107" s="264" t="n"/>
+      <c r="E107" s="423" t="n"/>
+      <c r="F107" s="423" t="n"/>
+      <c r="G107" s="423" t="n"/>
+      <c r="H107" s="423" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="263" t="n"/>
+      <c r="B108" s="262" t="n"/>
+      <c r="C108" s="262" t="n"/>
+      <c r="D108" s="264" t="n"/>
+      <c r="E108" s="423" t="n"/>
+      <c r="F108" s="423" t="n"/>
+      <c r="G108" s="423" t="n"/>
+      <c r="H108" s="423" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="263" t="n"/>
+      <c r="B109" s="262" t="n"/>
+      <c r="C109" s="262" t="n"/>
+      <c r="D109" s="264" t="n"/>
+      <c r="E109" s="423" t="n"/>
+      <c r="F109" s="423" t="n"/>
+      <c r="G109" s="423" t="n"/>
+      <c r="H109" s="423" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="263" t="n"/>
+      <c r="B110" s="262" t="n"/>
+      <c r="C110" s="262" t="n"/>
+      <c r="D110" s="264" t="n"/>
+      <c r="E110" s="423" t="n"/>
+      <c r="F110" s="423" t="n"/>
+      <c r="G110" s="423" t="n"/>
+      <c r="H110" s="423" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="263" t="n"/>
+      <c r="B111" s="262" t="n"/>
+      <c r="C111" s="262" t="n"/>
+      <c r="D111" s="264" t="n"/>
+      <c r="E111" s="423" t="n"/>
+      <c r="F111" s="423" t="n"/>
+      <c r="G111" s="423" t="n"/>
+      <c r="H111" s="423" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="263" t="n"/>
+      <c r="B112" s="262" t="n"/>
+      <c r="C112" s="262" t="n"/>
+      <c r="D112" s="264" t="n"/>
+      <c r="E112" s="423" t="n"/>
+      <c r="F112" s="423" t="n"/>
+      <c r="G112" s="423" t="n"/>
+      <c r="H112" s="423" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="263" t="n"/>
+      <c r="B113" s="262" t="n"/>
+      <c r="C113" s="262" t="n"/>
+      <c r="D113" s="264" t="n"/>
+      <c r="E113" s="423" t="n"/>
+      <c r="F113" s="423" t="n"/>
+      <c r="G113" s="423" t="n"/>
+      <c r="H113" s="423" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="263" t="n"/>
+      <c r="B114" s="262" t="n"/>
+      <c r="C114" s="262" t="n"/>
+      <c r="D114" s="264" t="n"/>
+      <c r="E114" s="423" t="n"/>
+      <c r="F114" s="423" t="n"/>
+      <c r="G114" s="423" t="n"/>
+      <c r="H114" s="423" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="263" t="n"/>
+      <c r="B115" s="262" t="n"/>
+      <c r="C115" s="262" t="n"/>
+      <c r="D115" s="264" t="n"/>
+      <c r="E115" s="423" t="n"/>
+      <c r="F115" s="423" t="n"/>
+      <c r="G115" s="423" t="n"/>
+      <c r="H115" s="423" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="263" t="n"/>
+      <c r="B116" s="262" t="n"/>
+      <c r="C116" s="262" t="n"/>
+      <c r="D116" s="264" t="n"/>
+      <c r="E116" s="423" t="n"/>
+      <c r="F116" s="423" t="n"/>
+      <c r="G116" s="423" t="n"/>
+      <c r="H116" s="423" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="263" t="n"/>
+      <c r="B117" s="262" t="n"/>
+      <c r="C117" s="262" t="n"/>
+      <c r="D117" s="264" t="n"/>
+      <c r="E117" s="423" t="n"/>
+      <c r="F117" s="423" t="n"/>
+      <c r="G117" s="423" t="n"/>
+      <c r="H117" s="423" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="263" t="n"/>
+      <c r="B118" s="262" t="n"/>
+      <c r="C118" s="262" t="n"/>
+      <c r="D118" s="264" t="n"/>
+      <c r="E118" s="423" t="n"/>
+      <c r="F118" s="423" t="n"/>
+      <c r="G118" s="423" t="n"/>
+      <c r="H118" s="423" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="263" t="n"/>
+      <c r="B119" s="262" t="n"/>
+      <c r="C119" s="262" t="n"/>
+      <c r="D119" s="264" t="n"/>
+      <c r="E119" s="423" t="n"/>
+      <c r="F119" s="423" t="n"/>
+      <c r="G119" s="423" t="n"/>
+      <c r="H119" s="423" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="263" t="n"/>
+      <c r="B120" s="262" t="n"/>
+      <c r="C120" s="262" t="n"/>
+      <c r="D120" s="264" t="n"/>
+      <c r="E120" s="423" t="n"/>
+      <c r="F120" s="423" t="n"/>
+      <c r="G120" s="423" t="n"/>
+      <c r="H120" s="423" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="263" t="n"/>
+      <c r="B121" s="262" t="n"/>
+      <c r="C121" s="262" t="n"/>
+      <c r="D121" s="264" t="n"/>
+      <c r="E121" s="423" t="n"/>
+      <c r="F121" s="423" t="n"/>
+      <c r="G121" s="423" t="n"/>
+      <c r="H121" s="423" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="263" t="n"/>
+      <c r="B122" s="262" t="n"/>
+      <c r="C122" s="262" t="n"/>
+      <c r="D122" s="264" t="n"/>
+      <c r="E122" s="423" t="n"/>
+      <c r="F122" s="423" t="n"/>
+      <c r="G122" s="423" t="n"/>
+      <c r="H122" s="423" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="262" t="n"/>
+      <c r="B123" s="262" t="inlineStr">
+        <is>
+          <t>TOTAL TIPS PASSED THROUGH</t>
+        </is>
+      </c>
+      <c r="C123" s="262" t="n"/>
+      <c r="D123" s="264">
+        <f>SUM(D63:D122)</f>
+        <v/>
+      </c>
+      <c r="E123" s="423" t="n"/>
+      <c r="F123" s="423" t="n"/>
+      <c r="G123" s="423" t="n"/>
+      <c r="H123" s="423" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="262" t="inlineStr">
+        <is>
+          <t>Customer tips collected &amp; handed to staff. Excluded from P&amp;L — nets to zero (received = paid).</t>
+        </is>
+      </c>
+      <c r="B124" s="262" t="n"/>
+      <c r="C124" s="262" t="n"/>
+      <c r="D124" s="262" t="n"/>
+      <c r="E124" s="423" t="n"/>
+      <c r="F124" s="423" t="n"/>
+      <c r="G124" s="423" t="n"/>
+      <c r="H124" s="423" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="423" t="n"/>
+      <c r="B125" s="423" t="n"/>
+      <c r="C125" s="423" t="n"/>
+      <c r="D125" s="423" t="n"/>
+      <c r="E125" s="423" t="n"/>
+      <c r="F125" s="423" t="n"/>
+      <c r="G125" s="423" t="n"/>
+      <c r="H125" s="423" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="423" t="inlineStr">
         <is>
           <t>── CASH RECONCILIATION (15 Jun 2026) ──</t>
         </is>
       </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="B126" s="423" t="n"/>
+      <c r="C126" s="423" t="n"/>
+      <c r="D126" s="423" t="n"/>
+      <c r="E126" s="423" t="n"/>
+      <c r="F126" s="423" t="n"/>
+      <c r="G126" s="423" t="n"/>
+      <c r="H126" s="423" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="423" t="inlineStr">
         <is>
           <t>Actual restaurant cash on hand</t>
         </is>
       </c>
-      <c r="D97" s="228" t="n">
+      <c r="B127" s="423" t="n"/>
+      <c r="C127" s="423" t="n"/>
+      <c r="D127" s="442" t="n">
         <v>20283</v>
       </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="E127" s="423" t="n"/>
+      <c r="F127" s="423" t="n"/>
+      <c r="G127" s="423" t="n"/>
+      <c r="H127" s="423" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="423" t="inlineStr">
         <is>
           <t>Adjustment: restaurant cash added to tips + Mercado Pago commission (vs running estimate)</t>
         </is>
       </c>
-      <c r="D98" s="228" t="n">
+      <c r="B128" s="423" t="n"/>
+      <c r="C128" s="423" t="n"/>
+      <c r="D128" s="442" t="n">
         <v>-165</v>
       </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="E128" s="423" t="n"/>
+      <c r="F128" s="423" t="n"/>
+      <c r="G128" s="423" t="n"/>
+      <c r="H128" s="423" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="423" t="inlineStr">
         <is>
           <t>Reconciled to physical count provided by Reddy. $20,283 is net of MP % deductions.</t>
         </is>
       </c>
+      <c r="B129" s="423" t="n"/>
+      <c r="C129" s="423" t="n"/>
+      <c r="D129" s="423" t="n"/>
+      <c r="E129" s="423" t="n"/>
+      <c r="F129" s="423" t="n"/>
+      <c r="G129" s="423" t="n"/>
+      <c r="H129" s="423" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -57394,7 +57832,7 @@
     <row r="24">
       <c r="A24" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Dairy</t>
+          <t>Utilities/Electricity</t>
         </is>
       </c>
       <c r="B24" s="437">
@@ -57424,7 +57862,7 @@
     <row r="25">
       <c r="A25" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Bread</t>
+          <t>Ingredients - Dairy</t>
         </is>
       </c>
       <c r="B25" s="437">
@@ -57454,7 +57892,7 @@
     <row r="26">
       <c r="A26" s="439" t="inlineStr">
         <is>
-          <t>Supplies/Other</t>
+          <t>Ingredients - Bread</t>
         </is>
       </c>
       <c r="B26" s="437">
@@ -57484,7 +57922,7 @@
     <row r="27">
       <c r="A27" s="439" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Supplies/Other</t>
         </is>
       </c>
       <c r="B27" s="437">
@@ -57514,7 +57952,7 @@
     <row r="28">
       <c r="A28" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Meat &amp; Fish</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B28" s="437">
@@ -57544,7 +57982,7 @@
     <row r="29">
       <c r="A29" s="439" t="inlineStr">
         <is>
-          <t>Packaging/Disposables</t>
+          <t>Ingredients - Meat &amp; Fish</t>
         </is>
       </c>
       <c r="B29" s="437">
@@ -57574,7 +58012,7 @@
     <row r="30">
       <c r="A30" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Gas</t>
+          <t>Packaging/Disposables</t>
         </is>
       </c>
       <c r="B30" s="437">
@@ -57604,7 +58042,7 @@
     <row r="31">
       <c r="A31" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Fruit</t>
+          <t>Utilities/Gas</t>
         </is>
       </c>
       <c r="B31" s="437">
@@ -57634,7 +58072,7 @@
     <row r="32">
       <c r="A32" s="439" t="inlineStr">
         <is>
-          <t>Kitchen Supplies</t>
+          <t>Ingredients - Fruit</t>
         </is>
       </c>
       <c r="B32" s="437">
@@ -57664,7 +58102,7 @@
     <row r="33">
       <c r="A33" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Internet</t>
+          <t>Kitchen Supplies</t>
         </is>
       </c>
       <c r="B33" s="437">
@@ -57694,7 +58132,7 @@
     <row r="34">
       <c r="A34" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Other</t>
+          <t>Utilities/Internet</t>
         </is>
       </c>
       <c r="B34" s="437">
@@ -57724,7 +58162,7 @@
     <row r="35">
       <c r="A35" s="439" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Ingredients - Other</t>
         </is>
       </c>
       <c r="B35" s="437">
@@ -57754,7 +58192,7 @@
     <row r="36">
       <c r="A36" s="439" t="inlineStr">
         <is>
-          <t>Software/Subscription</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="B36" s="437">
@@ -57784,7 +58222,7 @@
     <row r="37">
       <c r="A37" s="439" t="inlineStr">
         <is>
-          <t>Staff - Advance</t>
+          <t>Software/Subscription</t>
         </is>
       </c>
       <c r="B37" s="437">
@@ -57814,7 +58252,7 @@
     <row r="38">
       <c r="A38" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Desserts</t>
+          <t>Staff - Advance</t>
         </is>
       </c>
       <c r="B38" s="437">
@@ -57844,7 +58282,7 @@
     <row r="39">
       <c r="A39" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Eggs</t>
+          <t>Ingredients - Desserts</t>
         </is>
       </c>
       <c r="B39" s="437">
@@ -57874,7 +58312,7 @@
     <row r="40">
       <c r="A40" s="439" t="inlineStr">
         <is>
-          <t>Staff - Propinas</t>
+          <t>Ingredients - Eggs</t>
         </is>
       </c>
       <c r="B40" s="437">
@@ -57902,25 +58340,25 @@
       <c r="L40" s="433" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="436" t="inlineStr">
-        <is>
-          <t>TOTAL EXPENSES</t>
-        </is>
-      </c>
-      <c r="B41" s="438">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
-        <v/>
-      </c>
-      <c r="C41" s="438">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
-        <v/>
-      </c>
-      <c r="D41" s="438">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
-        <v/>
-      </c>
-      <c r="E41" s="438">
-        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,8,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,9,1))</f>
+      <c r="A41" s="439" t="inlineStr">
+        <is>
+          <t>Staff - Propinas</t>
+        </is>
+      </c>
+      <c r="B41" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
+        <v/>
+      </c>
+      <c r="C41" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
+        <v/>
+      </c>
+      <c r="D41" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
+        <v/>
+      </c>
+      <c r="E41" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,8,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,9,1))</f>
         <v/>
       </c>
       <c r="F41" s="433" t="n"/>
@@ -57934,23 +58372,23 @@
     <row r="42">
       <c r="A42" s="436" t="inlineStr">
         <is>
-          <t>NET PROFIT / LOSS</t>
+          <t>TOTAL EXPENSES</t>
         </is>
       </c>
       <c r="B42" s="438">
-        <f>B4-B41</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,5,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,6,1))</f>
         <v/>
       </c>
       <c r="C42" s="438">
-        <f>C4-C41</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,6,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,7,1))</f>
         <v/>
       </c>
       <c r="D42" s="438">
-        <f>D4-D41</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,7,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,8,1))</f>
         <v/>
       </c>
       <c r="E42" s="438">
-        <f>E4-E41</f>
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,8,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,9,1))</f>
         <v/>
       </c>
       <c r="F42" s="433" t="n"/>
@@ -57962,11 +58400,27 @@
       <c r="L42" s="433" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="433" t="n"/>
-      <c r="B43" s="433" t="n"/>
-      <c r="C43" s="433" t="n"/>
-      <c r="D43" s="433" t="n"/>
-      <c r="E43" s="433" t="n"/>
+      <c r="A43" s="436" t="inlineStr">
+        <is>
+          <t>NET PROFIT / LOSS</t>
+        </is>
+      </c>
+      <c r="B43" s="438">
+        <f>B4-B42</f>
+        <v/>
+      </c>
+      <c r="C43" s="438">
+        <f>C4-C42</f>
+        <v/>
+      </c>
+      <c r="D43" s="438">
+        <f>D4-D42</f>
+        <v/>
+      </c>
+      <c r="E43" s="438">
+        <f>E4-E42</f>
+        <v/>
+      </c>
       <c r="F43" s="433" t="n"/>
       <c r="G43" s="433" t="n"/>
       <c r="H43" s="433" t="n"/>

</xml_diff>

<commit_message>
added few more fixes
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -23275,9 +23275,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">

</xml_diff>

<commit_message>
updated yesterday and todays details
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -10262,45 +10262,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>6645.0</v>
+        <v>3315.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>120.0</v>
+        <v>0.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>2960.0</v>
+        <v>3736.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>3685.0</v>
+        <v>-421.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.554552</v>
+        <v>-0.126998</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>14580.0</v>
+        <v>23090.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>14580.0</v>
+        <v>23090.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*(MONTH($B$8:$B$5000)=MONTH(TODAY()))*(YEAR($B$8:$B$5000)=YEAR(TODAY()))*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>72543.0</v>
+        <v>81053.0</v>
       </c>
       <c r="P6">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($H$8:$H$5000),$H$8:$H$5000,0))</f>
-        <v>9306.0</v>
+        <v>13382.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>5274.0</v>
+        <v>9708.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -15902,62 +15902,140 @@
       <c r="AB94" s="324" t="n"/>
     </row>
     <row r="95" ht="16.5" customHeight="1" s="331">
-      <c r="B95" s="34" t="n"/>
-      <c r="C95" s="47" t="n"/>
-      <c r="D95" s="48" t="n"/>
-      <c r="E95" s="49" t="n"/>
-      <c r="F95" s="50" t="n"/>
-      <c r="G95" s="51" t="n"/>
-      <c r="H95" s="52" t="n"/>
-      <c r="I95" s="53" t="n"/>
-      <c r="J95" s="54" t="n"/>
-      <c r="K95" s="55" t="n"/>
-      <c r="L95" s="18" t="n"/>
-      <c r="M95" s="21" t="n"/>
-      <c r="N95" s="56" t="n"/>
-      <c r="O95" s="57" t="n"/>
-      <c r="P95" s="58" t="n"/>
-      <c r="Q95" s="56" t="n"/>
-      <c r="R95" s="56" t="n"/>
-      <c r="S95" s="56" t="n"/>
-      <c r="T95" s="56" t="n"/>
-      <c r="U95" s="56" t="n"/>
-      <c r="V95" s="56" t="n"/>
-      <c r="W95" s="56" t="n"/>
-      <c r="X95" s="56" t="n"/>
-      <c r="Y95" s="56" t="n"/>
-      <c r="Z95" s="56" t="n"/>
-      <c r="AA95" s="56" t="n"/>
-      <c r="AB95" s="56" t="n"/>
+      <c r="B95" s="427" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C95" s="255" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D95" s="256" t="n">
+        <v>3140</v>
+      </c>
+      <c r="E95" s="49" t="n">
+        <v>2055</v>
+      </c>
+      <c r="F95" s="50">
+        <f>IFERROR(D95+E95+G95+U95+Y95,0)</f>
+        <v>5195.0</v>
+      </c>
+      <c r="G95" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B95,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B95+1))</f>
+        <v>340.0</v>
+      </c>
+      <c r="I95" s="259">
+        <f>IFERROR(F95-H95,0)</f>
+        <v>4855.0</v>
+      </c>
+      <c r="J95" s="260">
+        <f>IFERROR(I95/F95,0)</f>
+        <v>0.934552</v>
+      </c>
+      <c r="K95" s="254" t="n"/>
+      <c r="L95" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M95" s="291" t="n"/>
+      <c r="N95" s="292" t="n"/>
+      <c r="O95" s="293" t="n"/>
+      <c r="P95" s="294" t="n"/>
+      <c r="Q95" s="292" t="n"/>
+      <c r="R95" s="443">
+        <f>IFERROR(D95*$T$7,0)</f>
+        <v>127.48</v>
+      </c>
+      <c r="S95" s="292" t="n"/>
+      <c r="T95" s="292" t="n"/>
+      <c r="U95" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V95" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W95" s="292" t="n"/>
+      <c r="X95" s="292" t="n"/>
+      <c r="Y95" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z95" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA95" s="292" t="n"/>
+      <c r="AB95" s="292" t="n"/>
     </row>
     <row r="96" ht="16.5" customHeight="1" s="331">
-      <c r="B96" s="34" t="n"/>
-      <c r="C96" s="35" t="n"/>
-      <c r="D96" s="36" t="n"/>
-      <c r="E96" s="37" t="n"/>
-      <c r="F96" s="38" t="n"/>
-      <c r="G96" s="39" t="n"/>
-      <c r="H96" s="40" t="n"/>
-      <c r="I96" s="41" t="n"/>
-      <c r="J96" s="42" t="n"/>
-      <c r="K96" s="43" t="n"/>
-      <c r="L96" s="9" t="n"/>
-      <c r="M96" s="12" t="n"/>
-      <c r="N96" s="44" t="n"/>
-      <c r="O96" s="45" t="n"/>
-      <c r="P96" s="46" t="n"/>
-      <c r="Q96" s="44" t="n"/>
-      <c r="R96" s="44" t="n"/>
-      <c r="S96" s="44" t="n"/>
-      <c r="T96" s="44" t="n"/>
-      <c r="U96" s="44" t="n"/>
-      <c r="V96" s="44" t="n"/>
-      <c r="W96" s="44" t="n"/>
-      <c r="X96" s="44" t="n"/>
-      <c r="Y96" s="44" t="n"/>
-      <c r="Z96" s="44" t="n"/>
-      <c r="AA96" s="44" t="n"/>
-      <c r="AB96" s="44" t="n"/>
+      <c r="B96" s="427" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C96" s="270" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D96" s="271" t="n">
+        <v>1210</v>
+      </c>
+      <c r="E96" s="37" t="n">
+        <v>2105</v>
+      </c>
+      <c r="F96" s="38">
+        <f>IFERROR(D96+E96+G96+U96+Y96,0)</f>
+        <v>3315.0</v>
+      </c>
+      <c r="G96" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B96,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B96+1))</f>
+        <v>3736.0</v>
+      </c>
+      <c r="I96" s="274">
+        <f>IFERROR(F96-H96,0)</f>
+        <v>-421.0</v>
+      </c>
+      <c r="J96" s="275">
+        <f>IFERROR(I96/F96,0)</f>
+        <v>-0.126998</v>
+      </c>
+      <c r="K96" s="250" t="n"/>
+      <c r="L96" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M96" s="323" t="n"/>
+      <c r="N96" s="324" t="n"/>
+      <c r="O96" s="325" t="n"/>
+      <c r="P96" s="326" t="n"/>
+      <c r="Q96" s="324" t="n"/>
+      <c r="R96" s="428">
+        <f>IFERROR(D96*$T$7,0)</f>
+        <v>49.13</v>
+      </c>
+      <c r="S96" s="324" t="n"/>
+      <c r="T96" s="324" t="n"/>
+      <c r="U96" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V96" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W96" s="324" t="n"/>
+      <c r="X96" s="324" t="n"/>
+      <c r="Y96" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z96" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA96" s="324" t="n"/>
+      <c r="AB96" s="324" t="n"/>
     </row>
     <row r="97" ht="16.5" customHeight="1" s="331">
       <c r="B97" s="34" t="n"/>
@@ -23990,7 +24068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J665"/>
+  <dimension ref="A1:J673"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -52088,6 +52166,350 @@
       <c r="J665" s="423" t="inlineStr">
         <is>
           <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="B666" s="429" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C666" s="297" t="inlineStr">
+        <is>
+          <t>Pescado</t>
+        </is>
+      </c>
+      <c r="D666" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E666" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="F666" s="299" t="n">
+        <v>340</v>
+      </c>
+      <c r="G666" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H666" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I666" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J666" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="B667" s="429" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C667" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D667" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E667" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F667" s="299" t="n">
+        <v>1176</v>
+      </c>
+      <c r="G667" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H667" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I667" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J667" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="B668" s="429" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C668" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D668" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E668" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F668" s="299" t="n">
+        <v>340</v>
+      </c>
+      <c r="G668" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H668" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I668" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J668" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="B669" s="429" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C669" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D669" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E669" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F669" s="299" t="n">
+        <v>114</v>
+      </c>
+      <c r="G669" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H669" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I669" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J669" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="B670" s="429" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C670" s="297" t="inlineStr">
+        <is>
+          <t>Agua Natural</t>
+        </is>
+      </c>
+      <c r="D670" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E670" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Beverages</t>
+        </is>
+      </c>
+      <c r="F670" s="299" t="n">
+        <v>30</v>
+      </c>
+      <c r="G670" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H670" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I670" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J670" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="B671" s="429" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C671" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D671" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E671" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F671" s="299" t="n">
+        <v>70</v>
+      </c>
+      <c r="G671" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H671" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I671" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J671" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="B672" s="429" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C672" s="297" t="inlineStr">
+        <is>
+          <t>Pan Reales</t>
+        </is>
+      </c>
+      <c r="D672" s="298" t="inlineStr">
+        <is>
+          <t>Pan Reales</t>
+        </is>
+      </c>
+      <c r="E672" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F672" s="299" t="n">
+        <v>156</v>
+      </c>
+      <c r="G672" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H672" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I672" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J672" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="B673" s="429" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C673" s="297" t="inlineStr">
+        <is>
+          <t>Armando - salary</t>
+        </is>
+      </c>
+      <c r="D673" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E673" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F673" s="299" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G673" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H673" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I673" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J673" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
paid back to capital update
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5509,7 +5509,7 @@
         </is>
       </c>
       <c r="C147" s="268" t="n">
-        <v>20911.85</v>
+        <v>14911.85</v>
       </c>
       <c r="E147" s="286" t="inlineStr">
         <is>
@@ -5531,11 +5531,11 @@
         </is>
       </c>
       <c r="C149" s="444" t="n">
-        <v>-44392</v>
+        <v>-50392</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Cumulative repaid from operating cash (latest 13-Aug-2026 $11,504.00). Reduces advance owed &amp; Cash-on-Hand; NOT a P&amp;L expense.</t>
+          <t>Cumulative repaid from operating cash (latest 21-Aug-2026 $6,000.00). Reduces advance owed &amp; Cash-on-Hand; NOT a P&amp;L expense.</t>
         </is>
       </c>
     </row>
@@ -24043,9 +24043,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">

</xml_diff>

<commit_message>
updated todays and yesterdays details
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -10262,7 +10262,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3315.0</v>
+        <v>2060.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -10270,37 +10270,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3736.0</v>
+        <v>4809.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>-421.0</v>
+        <v>-2749.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>-0.126998</v>
+        <v>-1.334466</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>23090.0</v>
+        <v>25150.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>23090.0</v>
+        <v>25150.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*(MONTH($B$8:$B$5000)=MONTH(TODAY()))*(YEAR($B$8:$B$5000)=YEAR(TODAY()))*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>81053.0</v>
+        <v>83113.0</v>
       </c>
       <c r="P6">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($H$8:$H$5000),$H$8:$H$5000,0))</f>
-        <v>13382.0</v>
+        <v>18191.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>9708.0</v>
+        <v>6959.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -16038,33 +16038,72 @@
       <c r="AB96" s="324" t="n"/>
     </row>
     <row r="97" ht="16.5" customHeight="1" s="331">
-      <c r="B97" s="34" t="n"/>
-      <c r="C97" s="47" t="n"/>
-      <c r="D97" s="48" t="n"/>
-      <c r="E97" s="49" t="n"/>
-      <c r="F97" s="50" t="n"/>
-      <c r="G97" s="51" t="n"/>
-      <c r="H97" s="52" t="n"/>
-      <c r="I97" s="53" t="n"/>
-      <c r="J97" s="54" t="n"/>
-      <c r="K97" s="55" t="n"/>
-      <c r="L97" s="18" t="n"/>
-      <c r="M97" s="21" t="n"/>
-      <c r="N97" s="56" t="n"/>
-      <c r="O97" s="57" t="n"/>
-      <c r="P97" s="58" t="n"/>
-      <c r="Q97" s="56" t="n"/>
-      <c r="R97" s="56" t="n"/>
-      <c r="S97" s="56" t="n"/>
-      <c r="T97" s="56" t="n"/>
-      <c r="U97" s="56" t="n"/>
-      <c r="V97" s="56" t="n"/>
-      <c r="W97" s="56" t="n"/>
-      <c r="X97" s="56" t="n"/>
-      <c r="Y97" s="56" t="n"/>
-      <c r="Z97" s="56" t="n"/>
-      <c r="AA97" s="56" t="n"/>
-      <c r="AB97" s="56" t="n"/>
+      <c r="B97" s="427" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C97" s="255" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D97" s="256" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="49" t="n">
+        <v>1015</v>
+      </c>
+      <c r="F97" s="50">
+        <f>IFERROR(D97+E97+G97+U97+Y97,0)</f>
+        <v>2060.0</v>
+      </c>
+      <c r="G97" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B97,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B97+1))</f>
+        <v>4809.0</v>
+      </c>
+      <c r="I97" s="259">
+        <f>IFERROR(F97-H97,0)</f>
+        <v>-2749.0</v>
+      </c>
+      <c r="J97" s="260">
+        <f>IFERROR(I97/F97,0)</f>
+        <v>-1.334466</v>
+      </c>
+      <c r="K97" s="254" t="n"/>
+      <c r="L97" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M97" s="291" t="n"/>
+      <c r="N97" s="292" t="n"/>
+      <c r="O97" s="293" t="n"/>
+      <c r="P97" s="294" t="n"/>
+      <c r="Q97" s="292" t="n"/>
+      <c r="R97" s="443">
+        <f>IFERROR(D97*$T$7,0)</f>
+        <v>0.0</v>
+      </c>
+      <c r="S97" s="292" t="n"/>
+      <c r="T97" s="292" t="n"/>
+      <c r="U97" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V97" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W97" s="292" t="n"/>
+      <c r="X97" s="292" t="n"/>
+      <c r="Y97" s="443" t="n">
+        <v>1045</v>
+      </c>
+      <c r="Z97" s="443" t="n">
+        <v>19.86</v>
+      </c>
+      <c r="AA97" s="292" t="n"/>
+      <c r="AB97" s="292" t="n"/>
     </row>
     <row r="98" ht="16.5" customHeight="1" s="331">
       <c r="B98" s="34" t="n"/>
@@ -24043,9 +24082,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -24068,7 +24107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J673"/>
+  <dimension ref="A1:J679"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -52510,6 +52549,264 @@
       <c r="J673" s="423" t="inlineStr">
         <is>
           <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="B674" s="429" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C674" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D674" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E674" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F674" s="299" t="n">
+        <v>109</v>
+      </c>
+      <c r="G674" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H674" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I674" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J674" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="B675" s="429" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C675" s="297" t="inlineStr">
+        <is>
+          <t>Jhon - salary</t>
+        </is>
+      </c>
+      <c r="D675" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E675" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F675" s="299" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G675" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H675" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I675" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J675" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="B676" s="429" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C676" s="297" t="inlineStr">
+        <is>
+          <t>Duvi - salary</t>
+        </is>
+      </c>
+      <c r="D676" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E676" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F676" s="299" t="n">
+        <v>500</v>
+      </c>
+      <c r="G676" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H676" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I676" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J676" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="B677" s="429" t="n">
+        <v>46257</v>
+      </c>
+      <c r="C677" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables Abastos</t>
+        </is>
+      </c>
+      <c r="D677" s="298" t="inlineStr">
+        <is>
+          <t>Central de Abastos</t>
+        </is>
+      </c>
+      <c r="E677" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F677" s="299" t="n">
+        <v>2046</v>
+      </c>
+      <c r="G677" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H677" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I677" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J677" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="B678" s="429" t="n">
+        <v>46257</v>
+      </c>
+      <c r="C678" s="297" t="inlineStr">
+        <is>
+          <t>Basicos</t>
+        </is>
+      </c>
+      <c r="D678" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E678" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F678" s="299" t="n">
+        <v>1241</v>
+      </c>
+      <c r="G678" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H678" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I678" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J678" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="B679" s="429" t="n">
+        <v>46257</v>
+      </c>
+      <c r="C679" s="297" t="inlineStr">
+        <is>
+          <t>San Juan Jamon</t>
+        </is>
+      </c>
+      <c r="D679" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E679" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F679" s="299" t="n">
+        <v>188</v>
+      </c>
+      <c r="G679" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H679" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I679" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J679" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
         </is>
       </c>
     </row>

</xml_diff>